<commit_message>
Fix issues found when verifying the Excel workbook
- Keep the space in second-tier idea names
- Add a detailed analogs column to the cards sheet
- Size rows from each cell's font so wrapped text is not clipped
- Widen summary columns whose headers broke mid-word
- Unmerge the summary note and mention the coloured input columns
- Validate the 0-1 lookup values, use A4 paper on every sheet
- Derive weight cells from data/ideas.json and round half up like Excel
- Restore the comment author after the LibreOffice recalculation

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwfWDVGmm96bgMjE9dGnWg
</commit_message>
<xml_diff>
--- a/ideas-russia-2026.xlsx
+++ b/ideas-russia-2026.xlsx
@@ -18,7 +18,7 @@
     <sheet name="Источники" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Карточки!$A$1:$N$35</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Карточки!$A$1:$O$35</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Сводная!$4:$4</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Сводная!$A$4:$Q$38</definedName>
   </definedNames>
@@ -34,7 +34,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <authors>
-    <author>Unknown Author</author>
+    <author>Анализ</author>
   </authors>
   <commentList>
     <comment ref="A4" authorId="0">
@@ -150,12 +150,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1133" uniqueCount="697">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="724">
   <si>
     <t xml:space="preserve">Онлайн-сервисы для России: 34 идеи, которые можно сделать с Claude Code (срез на 20.10.2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">Синие ячейки — экспертные оценки, их можно менять (есть выпадающие списки). Балл, место и стоимость в рублях считаются формулами; веса — на листе «Веса и шкалы». Подробное описание каждой идеи — на листе «Карточки».</t>
+    <t xml:space="preserve">Синие ячейки и цветные столбцы «Тип», «Конкуренция в РФ», «Регуляторный риск» — экспертные оценки, их можно менять (в цветных столбцах — выпадающие списки). Балл, место и стоимость в рублях считаются формулами; веса — на листе «Веса и шкалы». Подробное описание каждой идеи — на листе «Карточки».</t>
   </si>
   <si>
     <t xml:space="preserve">Место</t>
@@ -758,6 +758,9 @@
     <t xml:space="preserve">Балл</t>
   </si>
   <si>
+    <t xml:space="preserve">Аналоги (подробно)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Что это</t>
   </si>
   <si>
@@ -782,6 +785,9 @@
     <t xml:space="preserve">Ссылки</t>
   </si>
   <si>
+    <t xml:space="preserve">NYT Games (Wordle, Connections, Strands, Spelling Bee)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Каждый день выходят 4–5 коротких головоломок на 2–5 минут. Угадать слово из 5 букв. Разложить 16 слов на 4 скрытые группы («Связи»). Найти слова в сетке букв. Собрать как можно больше слов из 7 букв («Пчела»). Задания одинаковые для всех, поэтому результат можно сравнить с друзьями и поделиться им.</t>
   </si>
   <si>
@@ -830,6 +836,9 @@
     <t xml:space="preserve">https://www.jackboxgames.com/how-to</t>
   </si>
   <si>
+    <t xml:space="preserve">Infinite Craft (neal.fun)</t>
+  </si>
+  <si>
     <t xml:space="preserve">На старте есть 4 элемента: вода, огонь, земля, воздух. Соединяешь любые два, и нейросеть придумывает результат: огонь + вода = пар → … → «Кощей Бессмертный», «Пятиэтажка», «Ипотека». Комбинаций бесконечно много, а «первое в мире открытие» отмечается в игре.</t>
   </si>
   <si>
@@ -878,6 +887,9 @@
     <t xml:space="preserve">https://naked-science.ru/article/media/onlaine-game-geoguessr</t>
   </si>
   <si>
+    <t xml:space="preserve">Homescapes, Merge Mansion, Travel Town</t>
+  </si>
+  <si>
     <t xml:space="preserve">Соединяешь одинаковые предметы (2 кирпича → стена, 2 куска обоев → рулон) и так ремонтируешь советскую квартиру или дачу: ковёр на стене, сервант с хрусталём, телевизор «Рубин». Сюжет держится на историях соседей по подъезду.</t>
   </si>
   <si>
@@ -899,6 +911,9 @@
     <t xml:space="preserve">Самая дорогая из игровых идей: нужны регулярные обновления контента и тонкий баланс экономики. Без удержания игроков денег не будет.</t>
   </si>
   <si>
+    <t xml:space="preserve">Cal AI, одно из самых быстрорастущих приложений 2024–2025 годов</t>
+  </si>
+  <si>
     <t xml:space="preserve">Фотографируешь тарелку, приложение распознаёт блюдо и оценивает калории и БЖУ. Плюс дневник, цели и вес.</t>
   </si>
   <si>
@@ -921,6 +936,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.rustore.ru/catalog/app/com.nutrisync.advanced</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Timeleft (275 городов в 62 странах)</t>
   </si>
   <si>
     <t xml:space="preserve">Проходишь психологический тест. В выбранный день алгоритм собирает в ресторане стол из 6 подходящих друг другу людей. Это не свидания, а знакомство с новыми друзьями (Tasting Table).</t>
@@ -948,6 +966,9 @@
 https://daily.afisha.ru/archive/gorod/archive/behind-stay-hungry/</t>
   </si>
   <si>
+    <t xml:space="preserve">StoryWorth, Remento, Storii</t>
+  </si>
+  <si>
     <t xml:space="preserve">Раз в неделю маме, папе или бабушке приходит вопрос: «Как вы познакомились с дедушкой?», «Каким был ваш первый рабочий день?». Отвечать можно голосом, сервис расшифрует запись и бережно отредактирует. Через год получается печатная книга с фотографиями (Storii).</t>
   </si>
   <si>
@@ -970,6 +991,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://storii.com/blog/storyworth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joy Calls, Meela, CallieCare (США)</t>
   </si>
   <si>
     <t xml:space="preserve">В условленное время AI-голос звонит пожилому человеку на обычный телефон, даже кнопочный. Разговаривает о жизни, напоминает о лекарствах, помнит прошлые беседы. Семье приходит короткий отчёт: «настроение хорошее, жаловалась на давление, просила позвонить внучке» (Joy Calls, Meela).</t>
@@ -998,6 +1022,9 @@
 https://rozetked.me/index.php/news/47910-analitika-bol-she-poloviny-rossiyan-ispol-zuyut-ii-servisy-cifrovoy-zaschity</t>
   </si>
   <si>
+    <t xml:space="preserve">HelloChinese, SuperChinese + Praktika, Speak</t>
+  </si>
+  <si>
     <t xml:space="preserve">Приложение в духе Duolingo, но для китайского и для русскоязычных. Уроки HSK 1–4, тренажёр тонов с графиком высоты твоего голоса, разговорные сценки с AI («поторгуйся с поставщиком на выставке в Гуанчжоу»).</t>
   </si>
   <si>
@@ -1022,6 +1049,9 @@
     <t xml:space="preserve">https://apps.apple.com/us/app/%D0%BA%D0%B8%D1%82%D0%B0%D0%B9%D1%81%D0%BA%D0%B8%D0%B9-%D1%8F%D0%B7%D1%8B%D0%BA-%D1%81-%D0%BB%D0%B0%D0%BE%D1%88%D0%B8/id1510215770?l=ru</t>
   </si>
   <si>
+    <t xml:space="preserve">Yoodli, Google Interview Warmup</t>
+  </si>
+  <si>
     <t xml:space="preserve">AI голосом проводит собеседование под конкретную вакансию с hh.ru и задаёт уточняющие вопросы. Потом разбирает ответы: слова-паразиты, структура, темп, что улучшить. Режимы: собеседование, питч инвестору, разговор о повышении, защита диплома.</t>
   </si>
   <si>
@@ -1043,6 +1073,9 @@
     <t xml:space="preserve">Нельзя превращать продукт в «подсказчик на реальном собеседовании».</t>
   </si>
   <si>
+    <t xml:space="preserve">EssayGrader, Gauth/Photomath</t>
+  </si>
+  <si>
     <t xml:space="preserve">Школьник загружает фото или текст сочинения либо решения из второй части. Через 1–2 минуты получает оценку по критериям ФИПИ, разбор каждой ошибки и задание «исправь сам».</t>
   </si>
   <si>
@@ -1067,6 +1100,9 @@
     <t xml:space="preserve">https://yandex.cloud/ru/cases/aipushkin</t>
   </si>
   <si>
+    <t xml:space="preserve">MagicSchool AI, Brisk</t>
+  </si>
+  <si>
     <t xml:space="preserve">Учитель вводит «7 класс, тема "Пётр I"» и получает план урока по ФОП, рабочий лист трёх уровней сложности, тест и презентацию. Помощник проверяет диктанты по фото, пишет характеристики и отчёты.</t>
   </si>
   <si>
@@ -1088,6 +1124,9 @@
     <t xml:space="preserve">https://developers.sber.ru/help/gigachat-api/ai-for-teachers</t>
   </si>
   <si>
+    <t xml:space="preserve">TurboTenant, Avail, Landlord Studio</t>
+  </si>
+  <si>
     <t xml:space="preserve">Всё для сдачи квартиры в одном месте. Договор по шаблону для РФ. Акт приёма-передачи с фото. Напоминания и ссылки на оплату через СБП. Показания счётчиков и учёт ЖКУ. Чеки самозанятого (налог 4%). Проверка арендатора по открытым сервисам: недействительный паспорт, долги у ФССП. Расчёт залога при выезде.</t>
   </si>
   <si>
@@ -1136,6 +1175,9 @@
     <t xml:space="preserve">https://pravoved.ru/documents/new/claim/</t>
   </si>
   <si>
+    <t xml:space="preserve">Upsolve (США, некоммерческий сервис самостоятельного банкротства)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Человек с долгами отвечает на вопросы, и сервис говорит, подходит ли ему бесплатное внесудебное банкротство через МФЦ. Условия: долг от 25 тыс. до 1 млн ₽, оконченное исполнительное производство (разбор). Затем сервис собирает список кредиторов, заполняет заявление и ведёт по шагам. Если МФЦ не подходит, объясняет реструктуризацию и судебное банкротство и передаёт проверенному юристу.</t>
   </si>
   <si>
@@ -1157,6 +1199,9 @@
     <t xml:space="preserve">https://vitvet.com/articles/bankrotstvo/vnesudebnoe_bankrotstvo_mfc/</t>
   </si>
   <si>
+    <t xml:space="preserve">entitledto (Великобритания), benefits screeners (США)</t>
+  </si>
+  <si>
     <t xml:space="preserve">10–15 вопросов о семье, доходе и регионе. На выходе — все федеральные, региональные и муниципальные выплаты, льготы и налоговые вычеты, на которые человек имеет право, с суммами и пошаговой инструкцией. Плюс уведомления, когда правила меняются.</t>
   </si>
   <si>
@@ -1178,6 +1223,9 @@
     <t xml:space="preserve">https://finuslugi.ru/navigator/kak-ehto-rabotaet/stat_semeynaya-nalogovaya-vyplata-v-2026-godu</t>
   </si>
   <si>
+    <t xml:space="preserve">Wanderlog, Mindtrip, Layla</t>
+  </si>
+  <si>
     <t xml:space="preserve">Пишешь: «5 дней в Казани и Свияжске, с ребёнком 7 лет, бюджет 60 тыс.». Получаешь маршрут по дням с картой, временем в пути, ресторанами, ссылками на билеты и жильё, погодой и советами местных. Маршрут можно редактировать вместе с попутчиками и открыть без интернета.</t>
   </si>
   <si>
@@ -1202,6 +1250,9 @@
     <t xml:space="preserve">https://workspace.ru/cases/puteshestviya-po-rossii-ot-neyroseti/</t>
   </si>
   <si>
+    <t xml:space="preserve">Autio, GuideAlong (США)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Едешь в поезде «Москва — Казань» или по трассе М-12, а приложение по GPS рассказывает о том, что сейчас за окном: город, река, история, легенды, «через 10 минут — мост через Волгу». Работает без интернета, контент скачивается заранее.</t>
   </si>
   <si>
@@ -1265,6 +1316,9 @@
     <t xml:space="preserve">https://www.rustore.ru/catalog/app/ru.dacha.app</t>
   </si>
   <si>
+    <t xml:space="preserve">Mealime / Eat This Much + Flipp</t>
+  </si>
+  <si>
     <t xml:space="preserve">Указываешь состав семьи, вкусы, бюджет и ближайшие магазины. Сервис собирает меню на неделю из того, что сейчас по акции, выдаёт список покупок и делает один заказ в доставку. Учитывает, что уже лежит в холодильнике (по чекам).</t>
   </si>
   <si>
@@ -1286,6 +1340,9 @@
     <t xml:space="preserve">https://t-j.ru/discount-aggregators/</t>
   </si>
   <si>
+    <t xml:space="preserve">Goodcall, Slang.ai, Rosie</t>
+  </si>
+  <si>
     <t xml:space="preserve">AI круглосуточно отвечает на звонки салона, клиники или автосервиса. Записывает клиентов в YCLIENTS, Altegio или Dikidi, переносит записи, отвечает на вопросы о ценах, передаёт итог в CRM.</t>
   </si>
   <si>
@@ -1353,6 +1410,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://lifehacker.ru/yousician-guitar/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прямых аналогов нет</t>
   </si>
   <si>
     <t xml:space="preserve">Семья подключает пожилого родственника (заранее и с его согласия). Раз в 1–2 недели ему приходит безопасная учебная «атака»: звонок AI-голосом «из службы безопасности банка», «из полиции», «ваш сын попал в ДТП», «подтвердите код с Госуслуг». Если человек «попался», разговор мягко останавливается: «Это была тренировка от вашей дочери. Вот три признака, по которым можно было распознать обман». Семья видит прогресс, сценарии обновляются под новые схемы. Дополнительная функция: перешли подозрительное голосовое сообщение, и сервис оценит, не подделка ли это.</t>
@@ -1403,6 +1463,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://rg.ru/post/kak-proverit-nachisleniia-za-kommunalnye-uslugi-i-ne-pereplatit-za-zhkh.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Частичный аналог: проверка смет «Вс на стройку»</t>
   </si>
   <si>
     <t xml:space="preserve">Второй пилот ремонта на стороне заказчика:
@@ -1434,6 +1497,9 @@
     <t xml:space="preserve">https://spark.ru/startup/vs-na-strojku/blog/350477/sdelal-servis-kotorij-proveryaet-smeti-na-remont-za-pervuyu-nedelyu-nashli-pereplat-na-1-5-milliona-rublej</t>
   </si>
   <si>
+    <t xml:space="preserve">В мире — только исследования (Werewolf Arena от Google)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Онлайн-«Мафия», где недостающих игроков заменяют AI-персонажи со своими характерами: они блефуют, подозревают, защищаются. AI-ведущий озвучивает ночь и день. Режимы: «друзья + боты», «тренировка против AI», «AI-ведущий для офлайн-клуба».</t>
   </si>
   <si>
@@ -1458,6 +1524,9 @@
     <t xml:space="preserve">https://repo.ssau.ru/jspui/bitstream/123456789/31825/2/978-5-93424-903-9_2024_225-232.pdf</t>
   </si>
   <si>
+    <t xml:space="preserve">В мире — инди-эксперименты (CASE ZERO в альфе)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Каждый день новое дело: место преступления, улики, четыре подозреваемых. Ты допрашиваешь их текстом или голосом, AI-персонажи отвечают, путаются и скрывают. Предъявляешь обвинение, узнаёшь, прав ли ты, и сравниваешь результат с друзьями.</t>
   </si>
   <si>
@@ -1479,6 +1548,9 @@
     <t xml:space="preserve">https://dtf.ru/indie/5178362-rezhim-zhivye-podozrevaemye-v-case-zero</t>
   </si>
   <si>
+    <t xml:space="preserve">В мире есть только генераторы тостов</t>
+  </si>
+  <si>
     <t xml:space="preserve">Сервис готовит программу конкретного праздника: юбилей мамы, свадьба, выпускной. Гости заранее анонимно отвечают на 5 вопросов о виновнице торжества. Из ответов AI собирает викторину «Как хорошо вы знаете Галину?», тосты, конкурсы, плейлист и слайд-шоу из фото. В день праздника всё запускается на телевизоре, гости играют с телефонов. Детский режим — квест-поиск подарка по квартире с подсказками.</t>
   </si>
   <si>
@@ -1500,6 +1572,9 @@
     <t xml:space="preserve">Сезонность. Сарафанное радио лучше запускать через ведущих и ивент-агентства.</t>
   </si>
   <si>
+    <t xml:space="preserve">У врачей AI-ассистенты есть, у пациентов — нет</t>
+  </si>
+  <si>
     <t xml:space="preserve">Перед приёмом AI за 5 минут опрашивает пациента и делает одностраничную выписку для врача: жалобы, когда началось, какие лекарства принимает, какие анализы есть. На приёме, с согласия врача, записывает разговор. После приёма простыми словами объясняет, что сказал врач, напоминает о лекарствах и повторных анализах. Семейный режим — для пожилых родителей.</t>
   </si>
   <si>
@@ -1518,6 +1593,9 @@
     <t xml:space="preserve">Высокие. Данные о здоровье — особая категория. Есть граница с медицинским изделием: никаких диагнозов. Нужно согласие на запись.</t>
   </si>
   <si>
+    <t xml:space="preserve">Есть только универсальные суммаризаторы</t>
+  </si>
+  <si>
     <t xml:space="preserve">Бот, которого добавляют в чат класса или дома в Max. Раз в день он присылает выжимку: что решили, что купить, кто что должен и до какого срока. Ведёт голосования и учёт сборов («скинулись 21 из 28, вот список»), напоминает о делах. В домовых чатах собирает заявки в УК и совместные заказы мастера на весь подъезд.</t>
   </si>
   <si>
@@ -1536,6 +1614,9 @@
     <t xml:space="preserve">Зависимость от правил платформы Max. Конфиденциальность переписки.</t>
   </si>
   <si>
+    <t xml:space="preserve">Есть только классические агентства</t>
+  </si>
+  <si>
     <t xml:space="preserve">AI-голос звонит и пишет в компанию под видом клиента по сценарию: «хочу записаться на маникюр завтра», «сколько стоит замена ремня ГРМ». Проверяет, как отвечают сотрудники: скорость, вежливость, следование скрипту, предлагают ли допродажу. Присылает оценку и записи. Тот же механизм позволяет следить за публичными ценами и сроками конкурентов.</t>
   </si>
   <si>
@@ -1680,7 +1761,7 @@
     <t xml:space="preserve">Кластер</t>
   </si>
   <si>
-    <t xml:space="preserve">Продукты (в порядке запуска)</t>
+    <t xml:space="preserve">Продукты (→ — порядок запуска)</t>
   </si>
   <si>
     <t xml:space="preserve">Кто платит</t>
@@ -1879,19 +1960,19 @@
     <t xml:space="preserve">подросток «проживает день» хирурга, программиста или пилота. Минус: конкуренция с госпрограммами вроде «Билета в будущее».</t>
   </si>
   <si>
-    <t xml:space="preserve">Детектор голосовых дипфейковдля семей</t>
+    <t xml:space="preserve">Детектор голосовых дипфейков для семей</t>
   </si>
   <si>
     <t xml:space="preserve">Лучше сделать функцией внутри N01, а не отдельным продуктом.</t>
   </si>
   <si>
-    <t xml:space="preserve">Трекер детского сна с прогнозом «окна сна»(аналог Huckleberry)</t>
+    <t xml:space="preserve">Трекер детского сна с прогнозом «окна сна» (аналог Huckleberry)</t>
   </si>
   <si>
     <t xml:space="preserve">Ниша интересная, но спрос не проверял.</t>
   </si>
   <si>
-    <t xml:space="preserve">Простой планшет-лаунчер для бабушки с удалённым управлением детьми(аналог GrandPad)</t>
+    <t xml:space="preserve">Простой планшет-лаунчер для бабушки с удалённым управлением детьми (аналог GrandPad)</t>
   </si>
   <si>
     <t xml:space="preserve">Сильная синергия с M09 и N01, но нужно «железо».</t>
@@ -2440,7 +2521,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2449,8 +2530,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -2490,6 +2571,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -3145,11 +3230,12 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="30"/>
   </cols>
@@ -3159,26 +3245,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
@@ -3737,7 +3807,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="n">
         <f aca="false">RANK(E14,$E$5:$E$38,0)+COUNTIFS($E$5:$E$38,E14,$B$5:$B$38,"&lt;"&amp;B14)</f>
         <v>10</v>
@@ -4073,7 +4143,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="n">
         <f aca="false">RANK(E20,$E$5:$E$38,0)+COUNTIFS($E$5:$E$38,E20,$B$5:$B$38,"&lt;"&amp;B20)</f>
         <v>16</v>
@@ -4129,7 +4199,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="n">
         <f aca="false">RANK(E21,$E$5:$E$38,0)+COUNTIFS($E$5:$E$38,E21,$B$5:$B$38,"&lt;"&amp;B21)</f>
         <v>17</v>
@@ -4297,7 +4367,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="n">
         <f aca="false">RANK(E24,$E$5:$E$38,0)+COUNTIFS($E$5:$E$38,E24,$B$5:$B$38,"&lt;"&amp;B24)</f>
         <v>20</v>
@@ -4745,7 +4815,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="n">
         <f aca="false">RANK(E32,$E$5:$E$38,0)+COUNTIFS($E$5:$E$38,E32,$B$5:$B$38,"&lt;"&amp;B32)</f>
         <v>28</v>
@@ -4857,7 +4927,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="n">
         <f aca="false">RANK(E34,$E$5:$E$38,0)+COUNTIFS($E$5:$E$38,E34,$B$5:$B$38,"&lt;"&amp;B34)</f>
         <v>30</v>
@@ -4913,7 +4983,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="n">
         <f aca="false">RANK(E35,$E$5:$E$38,0)+COUNTIFS($E$5:$E$38,E35,$B$5:$B$38,"&lt;"&amp;B35)</f>
         <v>31</v>
@@ -5139,9 +5209,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:Q38"/>
-  <mergeCells count="1">
-    <mergeCell ref="A2:Q2"/>
-  </mergeCells>
   <conditionalFormatting sqref="E5:E38">
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -5246,7 +5313,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5261,7 +5328,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:N35"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -5270,12 +5337,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5321,8 +5389,11 @@
       <c r="N1" s="3" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="2" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="O1" s="3" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>36</v>
       </c>
@@ -5344,31 +5415,34 @@
         <v>40</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H2" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I2" s="9" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="J2" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K2" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="L2" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="M2" s="9" t="s">
-        <v>216</v>
-      </c>
-      <c r="N2" s="12" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N2" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="O2" s="12" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>79</v>
       </c>
@@ -5390,31 +5464,34 @@
         <v>81</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>218</v>
+        <v>81</v>
       </c>
       <c r="H3" s="9" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="J3" s="9" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="L3" s="9" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="M3" s="9" t="s">
-        <v>224</v>
-      </c>
-      <c r="N3" s="12" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="N3" s="9" t="s">
+        <v>226</v>
+      </c>
+      <c r="O3" s="12" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>63</v>
       </c>
@@ -5436,31 +5513,34 @@
         <v>65</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="I4" s="9" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="J4" s="9" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="L4" s="9" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="M4" s="9" t="s">
-        <v>232</v>
-      </c>
-      <c r="N4" s="12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>234</v>
+      </c>
+      <c r="N4" s="9" t="s">
+        <v>235</v>
+      </c>
+      <c r="O4" s="12" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>167</v>
       </c>
@@ -5482,31 +5562,34 @@
         <v>169</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>234</v>
+        <v>169</v>
       </c>
       <c r="H5" s="9" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="I5" s="9" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="J5" s="9" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="L5" s="9" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="M5" s="9" t="s">
-        <v>240</v>
-      </c>
-      <c r="N5" s="12" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>242</v>
+      </c>
+      <c r="N5" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="O5" s="12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
         <v>125</v>
       </c>
@@ -5528,28 +5611,31 @@
         <v>127</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="I6" s="9" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="J6" s="9" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="L6" s="9" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="M6" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="N6" s="12" t="s">
-        <v>233</v>
+        <v>251</v>
+      </c>
+      <c r="N6" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="O6" s="12" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5574,31 +5660,34 @@
         <v>105</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="J7" s="9" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>253</v>
+        <v>257</v>
       </c>
       <c r="L7" s="9" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="M7" s="9" t="s">
-        <v>255</v>
-      </c>
-      <c r="N7" s="12" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>259</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="O7" s="12" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
         <v>136</v>
       </c>
@@ -5620,31 +5709,34 @@
         <v>138</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="I8" s="9" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="J8" s="9" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="L8" s="9" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="M8" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="N8" s="12" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>268</v>
+      </c>
+      <c r="N8" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="O8" s="12" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
         <v>84</v>
       </c>
@@ -5666,31 +5758,34 @@
         <v>86</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="H9" s="9" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="I9" s="9" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="J9" s="9" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="L9" s="9" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="M9" s="9" t="s">
-        <v>271</v>
-      </c>
-      <c r="N9" s="12" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>277</v>
+      </c>
+      <c r="N9" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="O9" s="12" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="105" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
         <v>108</v>
       </c>
@@ -5712,28 +5807,31 @@
         <v>110</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="J10" s="9" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="L10" s="9" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="M10" s="9" t="s">
-        <v>279</v>
-      </c>
-      <c r="N10" s="12" t="s">
-        <v>280</v>
+        <v>286</v>
+      </c>
+      <c r="N10" s="9" t="s">
+        <v>287</v>
+      </c>
+      <c r="O10" s="12" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5758,28 +5856,31 @@
         <v>190</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="J11" s="9" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="L11" s="9" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="M11" s="9" t="s">
-        <v>287</v>
-      </c>
-      <c r="N11" s="12" t="s">
-        <v>288</v>
+        <v>295</v>
+      </c>
+      <c r="N11" s="9" t="s">
+        <v>296</v>
+      </c>
+      <c r="O11" s="12" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5804,31 +5905,34 @@
         <v>91</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="J12" s="9" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="L12" s="9" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="M12" s="9" t="s">
-        <v>295</v>
-      </c>
-      <c r="N12" s="12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>304</v>
+      </c>
+      <c r="N12" s="9" t="s">
+        <v>305</v>
+      </c>
+      <c r="O12" s="12" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
         <v>93</v>
       </c>
@@ -5850,28 +5954,31 @@
         <v>95</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>296</v>
+        <v>306</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>297</v>
+        <v>307</v>
       </c>
       <c r="I13" s="9" t="s">
-        <v>298</v>
+        <v>308</v>
       </c>
       <c r="J13" s="9" t="s">
-        <v>299</v>
+        <v>309</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="L13" s="9" t="s">
-        <v>301</v>
+        <v>311</v>
       </c>
       <c r="M13" s="9" t="s">
-        <v>302</v>
-      </c>
-      <c r="N13" s="12" t="s">
-        <v>303</v>
+        <v>312</v>
+      </c>
+      <c r="N13" s="9" t="s">
+        <v>313</v>
+      </c>
+      <c r="O13" s="12" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5896,31 +6003,34 @@
         <v>195</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>305</v>
+        <v>316</v>
       </c>
       <c r="I14" s="9" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="J14" s="9" t="s">
-        <v>307</v>
+        <v>318</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>233</v>
+        <v>319</v>
       </c>
       <c r="L14" s="9" t="s">
-        <v>308</v>
+        <v>236</v>
       </c>
       <c r="M14" s="9" t="s">
-        <v>309</v>
-      </c>
-      <c r="N14" s="12" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>320</v>
+      </c>
+      <c r="N14" s="9" t="s">
+        <v>321</v>
+      </c>
+      <c r="O14" s="12" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
         <v>98</v>
       </c>
@@ -5942,31 +6052,34 @@
         <v>100</v>
       </c>
       <c r="G15" s="9" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="J15" s="9" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="M15" s="9" t="s">
-        <v>317</v>
-      </c>
-      <c r="N15" s="12" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="131.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>329</v>
+      </c>
+      <c r="N15" s="9" t="s">
+        <v>330</v>
+      </c>
+      <c r="O15" s="12" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="144" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
         <v>45</v>
       </c>
@@ -5988,31 +6101,34 @@
         <v>47</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>319</v>
+        <v>47</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="J16" s="9" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="L16" s="9" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="M16" s="9" t="s">
-        <v>325</v>
-      </c>
-      <c r="N16" s="12" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>337</v>
+      </c>
+      <c r="N16" s="9" t="s">
+        <v>338</v>
+      </c>
+      <c r="O16" s="12" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="131.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
         <v>171</v>
       </c>
@@ -6034,28 +6150,31 @@
         <v>173</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>327</v>
+        <v>340</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>328</v>
+        <v>341</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>329</v>
+        <v>342</v>
       </c>
       <c r="J17" s="9" t="s">
-        <v>330</v>
+        <v>343</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>233</v>
+        <v>344</v>
       </c>
       <c r="L17" s="9" t="s">
-        <v>331</v>
+        <v>236</v>
       </c>
       <c r="M17" s="9" t="s">
-        <v>332</v>
-      </c>
-      <c r="N17" s="12" t="s">
-        <v>333</v>
+        <v>345</v>
+      </c>
+      <c r="N17" s="9" t="s">
+        <v>346</v>
+      </c>
+      <c r="O17" s="12" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6080,31 +6199,34 @@
         <v>177</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>334</v>
+        <v>348</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>335</v>
+        <v>349</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>336</v>
+        <v>350</v>
       </c>
       <c r="J18" s="9" t="s">
-        <v>337</v>
+        <v>351</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>233</v>
+        <v>352</v>
       </c>
       <c r="L18" s="9" t="s">
-        <v>338</v>
+        <v>236</v>
       </c>
       <c r="M18" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="N18" s="12" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>353</v>
+      </c>
+      <c r="N18" s="9" t="s">
+        <v>354</v>
+      </c>
+      <c r="O18" s="12" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
         <v>69</v>
       </c>
@@ -6126,31 +6248,34 @@
         <v>72</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>341</v>
+        <v>356</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
       <c r="J19" s="9" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
       <c r="M19" s="9" t="s">
-        <v>347</v>
-      </c>
-      <c r="N19" s="12" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>362</v>
+      </c>
+      <c r="N19" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="O19" s="12" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
         <v>147</v>
       </c>
@@ -6172,31 +6297,34 @@
         <v>149</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>349</v>
+        <v>365</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>350</v>
+        <v>366</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>351</v>
+        <v>367</v>
       </c>
       <c r="J20" s="9" t="s">
-        <v>352</v>
+        <v>368</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>353</v>
+        <v>369</v>
       </c>
       <c r="L20" s="9" t="s">
-        <v>354</v>
+        <v>370</v>
       </c>
       <c r="M20" s="9" t="s">
-        <v>355</v>
-      </c>
-      <c r="N20" s="12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>371</v>
+      </c>
+      <c r="N20" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="O20" s="12" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
         <v>179</v>
       </c>
@@ -6218,31 +6346,34 @@
         <v>181</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>356</v>
+        <v>181</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>357</v>
+        <v>373</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>358</v>
+        <v>374</v>
       </c>
       <c r="J21" s="9" t="s">
-        <v>359</v>
+        <v>375</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>233</v>
+        <v>376</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>360</v>
+        <v>236</v>
       </c>
       <c r="M21" s="9" t="s">
-        <v>361</v>
-      </c>
-      <c r="N21" s="12" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>377</v>
+      </c>
+      <c r="N21" s="9" t="s">
+        <v>378</v>
+      </c>
+      <c r="O21" s="12" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
         <v>152</v>
       </c>
@@ -6264,31 +6395,34 @@
         <v>154</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>363</v>
+        <v>154</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>364</v>
+        <v>380</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="J22" s="9" t="s">
-        <v>366</v>
+        <v>382</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>233</v>
+        <v>383</v>
       </c>
       <c r="L22" s="9" t="s">
-        <v>367</v>
+        <v>236</v>
       </c>
       <c r="M22" s="9" t="s">
-        <v>368</v>
-      </c>
-      <c r="N22" s="12" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>384</v>
+      </c>
+      <c r="N22" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="O22" s="12" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
         <v>131</v>
       </c>
@@ -6310,31 +6444,34 @@
         <v>134</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>370</v>
+        <v>387</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>371</v>
+        <v>388</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>372</v>
+        <v>389</v>
       </c>
       <c r="J23" s="9" t="s">
-        <v>373</v>
+        <v>390</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>233</v>
+        <v>391</v>
       </c>
       <c r="L23" s="9" t="s">
-        <v>374</v>
+        <v>236</v>
       </c>
       <c r="M23" s="9" t="s">
-        <v>375</v>
-      </c>
-      <c r="N23" s="12" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>392</v>
+      </c>
+      <c r="N23" s="9" t="s">
+        <v>393</v>
+      </c>
+      <c r="O23" s="12" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
         <v>197</v>
       </c>
@@ -6356,31 +6493,34 @@
         <v>199</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>377</v>
+        <v>395</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>378</v>
+        <v>396</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>379</v>
+        <v>397</v>
       </c>
       <c r="J24" s="9" t="s">
-        <v>380</v>
+        <v>398</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>381</v>
+        <v>399</v>
       </c>
       <c r="L24" s="9" t="s">
-        <v>382</v>
+        <v>400</v>
       </c>
       <c r="M24" s="9" t="s">
-        <v>383</v>
-      </c>
-      <c r="N24" s="12" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>401</v>
+      </c>
+      <c r="N24" s="9" t="s">
+        <v>402</v>
+      </c>
+      <c r="O24" s="12" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
         <v>141</v>
       </c>
@@ -6402,31 +6542,34 @@
         <v>144</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>385</v>
+        <v>144</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>386</v>
+        <v>404</v>
       </c>
       <c r="I25" s="9" t="s">
-        <v>387</v>
+        <v>405</v>
       </c>
       <c r="J25" s="9" t="s">
-        <v>388</v>
+        <v>406</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>389</v>
+        <v>407</v>
       </c>
       <c r="L25" s="9" t="s">
-        <v>390</v>
+        <v>408</v>
       </c>
       <c r="M25" s="9" t="s">
-        <v>391</v>
-      </c>
-      <c r="N25" s="12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>409</v>
+      </c>
+      <c r="N25" s="9" t="s">
+        <v>410</v>
+      </c>
+      <c r="O25" s="12" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
         <v>184</v>
       </c>
@@ -6448,31 +6591,34 @@
         <v>186</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>392</v>
+        <v>186</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>393</v>
+        <v>411</v>
       </c>
       <c r="I26" s="9" t="s">
-        <v>394</v>
+        <v>412</v>
       </c>
       <c r="J26" s="9" t="s">
-        <v>395</v>
+        <v>413</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>396</v>
+        <v>414</v>
       </c>
       <c r="L26" s="9" t="s">
-        <v>397</v>
+        <v>415</v>
       </c>
       <c r="M26" s="9" t="s">
-        <v>398</v>
-      </c>
-      <c r="N26" s="12" t="s">
-        <v>399</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="156.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>416</v>
+      </c>
+      <c r="N26" s="9" t="s">
+        <v>417</v>
+      </c>
+      <c r="O26" s="12" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="182.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>19</v>
       </c>
@@ -6494,31 +6640,34 @@
         <v>23</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>400</v>
+        <v>419</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>401</v>
+        <v>420</v>
       </c>
       <c r="I27" s="9" t="s">
-        <v>402</v>
+        <v>421</v>
       </c>
       <c r="J27" s="9" t="s">
-        <v>403</v>
+        <v>422</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>404</v>
+        <v>423</v>
       </c>
       <c r="L27" s="9" t="s">
-        <v>405</v>
+        <v>424</v>
       </c>
       <c r="M27" s="9" t="s">
-        <v>406</v>
-      </c>
-      <c r="N27" s="12" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>425</v>
+      </c>
+      <c r="N27" s="9" t="s">
+        <v>426</v>
+      </c>
+      <c r="O27" s="12" t="s">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
         <v>29</v>
       </c>
@@ -6540,31 +6689,34 @@
         <v>32</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>408</v>
+        <v>419</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>409</v>
+        <v>428</v>
       </c>
       <c r="I28" s="9" t="s">
-        <v>410</v>
+        <v>429</v>
       </c>
       <c r="J28" s="9" t="s">
-        <v>411</v>
+        <v>430</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>412</v>
+        <v>431</v>
       </c>
       <c r="L28" s="9" t="s">
-        <v>413</v>
+        <v>432</v>
       </c>
       <c r="M28" s="9" t="s">
-        <v>414</v>
-      </c>
-      <c r="N28" s="12" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="156.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>433</v>
+      </c>
+      <c r="N28" s="9" t="s">
+        <v>434</v>
+      </c>
+      <c r="O28" s="12" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="169.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
         <v>58</v>
       </c>
@@ -6586,31 +6738,34 @@
         <v>60</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>416</v>
+        <v>436</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>417</v>
+        <v>437</v>
       </c>
       <c r="I29" s="9" t="s">
-        <v>418</v>
+        <v>438</v>
       </c>
       <c r="J29" s="9" t="s">
-        <v>419</v>
+        <v>439</v>
       </c>
       <c r="K29" s="9" t="s">
-        <v>420</v>
+        <v>440</v>
       </c>
       <c r="L29" s="9" t="s">
-        <v>421</v>
+        <v>441</v>
       </c>
       <c r="M29" s="9" t="s">
-        <v>422</v>
-      </c>
-      <c r="N29" s="12" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>442</v>
+      </c>
+      <c r="N29" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="O29" s="12" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
         <v>74</v>
       </c>
@@ -6632,31 +6787,34 @@
         <v>76</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>425</v>
+        <v>446</v>
       </c>
       <c r="I30" s="9" t="s">
-        <v>426</v>
+        <v>447</v>
       </c>
       <c r="J30" s="9" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="K30" s="9" t="s">
-        <v>428</v>
+        <v>449</v>
       </c>
       <c r="L30" s="9" t="s">
-        <v>429</v>
+        <v>450</v>
       </c>
       <c r="M30" s="9" t="s">
-        <v>430</v>
-      </c>
-      <c r="N30" s="12" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>451</v>
+      </c>
+      <c r="N30" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="O30" s="12" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="80.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
         <v>114</v>
       </c>
@@ -6678,31 +6836,34 @@
         <v>116</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>432</v>
+        <v>454</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>433</v>
+        <v>455</v>
       </c>
       <c r="I31" s="9" t="s">
-        <v>434</v>
+        <v>456</v>
       </c>
       <c r="J31" s="9" t="s">
-        <v>233</v>
+        <v>457</v>
       </c>
       <c r="K31" s="9" t="s">
-        <v>435</v>
+        <v>236</v>
       </c>
       <c r="L31" s="9" t="s">
-        <v>436</v>
+        <v>458</v>
       </c>
       <c r="M31" s="9" t="s">
-        <v>437</v>
-      </c>
-      <c r="N31" s="12" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>459</v>
+      </c>
+      <c r="N31" s="9" t="s">
+        <v>460</v>
+      </c>
+      <c r="O31" s="12" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="131.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
         <v>52</v>
       </c>
@@ -6724,31 +6885,34 @@
         <v>55</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>439</v>
+        <v>462</v>
       </c>
       <c r="H32" s="9" t="s">
-        <v>440</v>
+        <v>463</v>
       </c>
       <c r="I32" s="9" t="s">
-        <v>441</v>
+        <v>464</v>
       </c>
       <c r="J32" s="9" t="s">
-        <v>442</v>
+        <v>465</v>
       </c>
       <c r="K32" s="9" t="s">
-        <v>443</v>
+        <v>466</v>
       </c>
       <c r="L32" s="9" t="s">
-        <v>444</v>
+        <v>467</v>
       </c>
       <c r="M32" s="9" t="s">
-        <v>445</v>
-      </c>
-      <c r="N32" s="12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>468</v>
+      </c>
+      <c r="N32" s="9" t="s">
+        <v>469</v>
+      </c>
+      <c r="O32" s="12" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
         <v>162</v>
       </c>
@@ -6770,31 +6934,34 @@
         <v>164</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>446</v>
+        <v>470</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>447</v>
+        <v>471</v>
       </c>
       <c r="I33" s="9" t="s">
-        <v>448</v>
+        <v>472</v>
       </c>
       <c r="J33" s="9" t="s">
-        <v>449</v>
+        <v>473</v>
       </c>
       <c r="K33" s="9" t="s">
-        <v>233</v>
+        <v>474</v>
       </c>
       <c r="L33" s="9" t="s">
-        <v>450</v>
+        <v>236</v>
       </c>
       <c r="M33" s="9" t="s">
-        <v>451</v>
-      </c>
-      <c r="N33" s="12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>475</v>
+      </c>
+      <c r="N33" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="O33" s="12" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
         <v>119</v>
       </c>
@@ -6816,31 +6983,34 @@
         <v>121</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>452</v>
+        <v>477</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>453</v>
+        <v>478</v>
       </c>
       <c r="I34" s="9" t="s">
-        <v>454</v>
+        <v>479</v>
       </c>
       <c r="J34" s="9" t="s">
-        <v>455</v>
+        <v>480</v>
       </c>
       <c r="K34" s="9" t="s">
-        <v>233</v>
+        <v>481</v>
       </c>
       <c r="L34" s="9" t="s">
-        <v>456</v>
+        <v>236</v>
       </c>
       <c r="M34" s="9" t="s">
-        <v>457</v>
-      </c>
-      <c r="N34" s="12" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="105.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>482</v>
+      </c>
+      <c r="N34" s="9" t="s">
+        <v>483</v>
+      </c>
+      <c r="O34" s="12" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="118.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
         <v>157</v>
       </c>
@@ -6862,32 +7032,35 @@
         <v>159</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>458</v>
+        <v>484</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>459</v>
+        <v>485</v>
       </c>
       <c r="I35" s="9" t="s">
-        <v>460</v>
+        <v>486</v>
       </c>
       <c r="J35" s="9" t="s">
-        <v>461</v>
+        <v>487</v>
       </c>
       <c r="K35" s="9" t="s">
-        <v>233</v>
+        <v>488</v>
       </c>
       <c r="L35" s="9" t="s">
-        <v>462</v>
+        <v>236</v>
       </c>
       <c r="M35" s="9" t="s">
-        <v>463</v>
-      </c>
-      <c r="N35" s="12" t="s">
-        <v>233</v>
+        <v>489</v>
+      </c>
+      <c r="N35" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="O35" s="12" t="s">
+        <v>236</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N35"/>
+  <autoFilter ref="A1:O35"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -6915,137 +7088,137 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>464</v>
+        <v>491</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>465</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
+      <c r="A2" s="13" t="s">
+        <v>492</v>
+      </c>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>466</v>
+        <v>493</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>467</v>
+        <v>494</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>468</v>
+        <v>495</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>469</v>
+        <v>496</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>470</v>
+        <v>497</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>471</v>
-      </c>
-      <c r="C6" s="13" t="n">
+        <v>498</v>
+      </c>
+      <c r="C6" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="15" t="n">
         <f aca="false">IF(SUM($C$6:$C$11)=0,0,C6/SUM($C$6:$C$11))</f>
         <v>0.25</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>472</v>
+        <v>499</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>473</v>
-      </c>
-      <c r="C7" s="13" t="n">
+        <v>500</v>
+      </c>
+      <c r="C7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="15" t="n">
         <f aca="false">IF(SUM($C$6:$C$11)=0,0,C7/SUM($C$6:$C$11))</f>
         <v>0.2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>474</v>
+        <v>501</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>475</v>
-      </c>
-      <c r="C8" s="13" t="n">
+        <v>502</v>
+      </c>
+      <c r="C8" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="15" t="n">
         <f aca="false">IF(SUM($C$6:$C$11)=0,0,C8/SUM($C$6:$C$11))</f>
         <v>0.2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>476</v>
+        <v>503</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>477</v>
-      </c>
-      <c r="C9" s="13" t="n">
+        <v>504</v>
+      </c>
+      <c r="C9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="15" t="n">
         <f aca="false">IF(SUM($C$6:$C$11)=0,0,C9/SUM($C$6:$C$11))</f>
         <v>0.15</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>478</v>
+        <v>505</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>479</v>
-      </c>
-      <c r="C10" s="13" t="n">
+        <v>506</v>
+      </c>
+      <c r="C10" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="15" t="n">
         <f aca="false">IF(SUM($C$6:$C$11)=0,0,C10/SUM($C$6:$C$11))</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>480</v>
+        <v>507</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>481</v>
-      </c>
-      <c r="C11" s="13" t="n">
+        <v>508</v>
+      </c>
+      <c r="C11" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="15" t="n">
         <f aca="false">IF(SUM($C$6:$C$11)=0,0,C11/SUM($C$6:$C$11))</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>482</v>
+        <v>509</v>
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">SUM(C6:C11)</f>
         <v>20</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="D12" s="16" t="n">
         <f aca="false">SUM(D6:D11)</f>
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="16" t="s">
-        <v>483</v>
+      <c r="A14" s="17" t="s">
+        <v>510</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7053,14 +7226,14 @@
         <v>15</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>484</v>
+        <v>511</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B16" s="13" t="n">
+      <c r="B16" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7068,7 +7241,7 @@
       <c r="A17" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B17" s="13" t="n">
+      <c r="B17" s="14" t="n">
         <v>0.75</v>
       </c>
     </row>
@@ -7076,15 +7249,15 @@
       <c r="A18" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="14" t="n">
         <v>0.5</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>485</v>
-      </c>
-      <c r="B19" s="13" t="n">
+        <v>512</v>
+      </c>
+      <c r="B19" s="14" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -7093,14 +7266,14 @@
         <v>16</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>486</v>
+        <v>513</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B23" s="13" t="n">
+      <c r="B23" s="14" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7108,7 +7281,7 @@
       <c r="A24" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="13" t="n">
+      <c r="B24" s="14" t="n">
         <v>0.6</v>
       </c>
     </row>
@@ -7116,34 +7289,34 @@
       <c r="A25" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="B25" s="13" t="n">
+      <c r="B25" s="14" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="16" t="s">
-        <v>487</v>
+      <c r="A28" s="17" t="s">
+        <v>514</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="17" t="s">
-        <v>488</v>
-      </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="17"/>
-      <c r="D29" s="17"/>
+      <c r="A29" s="18" t="s">
+        <v>515</v>
+      </c>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="16" t="s">
-        <v>489</v>
+      <c r="A31" s="17" t="s">
+        <v>516</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>490</v>
+        <v>517</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>491</v>
+        <v>518</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7151,17 +7324,17 @@
         <v>9</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>492</v>
+        <v>519</v>
       </c>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>493</v>
+        <v>520</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>494</v>
+        <v>521</v>
       </c>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
@@ -7171,7 +7344,7 @@
         <v>13</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>495</v>
+        <v>522</v>
       </c>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
@@ -7181,7 +7354,7 @@
         <v>14</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>496</v>
+        <v>523</v>
       </c>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
@@ -7191,7 +7364,7 @@
         <v>15</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>497</v>
+        <v>524</v>
       </c>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
@@ -7201,55 +7374,55 @@
         <v>16</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>498</v>
+        <v>525</v>
       </c>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="16" t="s">
-        <v>499</v>
+      <c r="A40" s="17" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="17" t="s">
-        <v>500</v>
-      </c>
-      <c r="B41" s="17"/>
-      <c r="C41" s="17"/>
-      <c r="D41" s="17"/>
+      <c r="A41" s="18" t="s">
+        <v>527</v>
+      </c>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
     </row>
     <row r="42" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="17" t="s">
-        <v>501</v>
-      </c>
-      <c r="B42" s="17"/>
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
+      <c r="A42" s="18" t="s">
+        <v>528</v>
+      </c>
+      <c r="B42" s="18"/>
+      <c r="C42" s="18"/>
+      <c r="D42" s="18"/>
     </row>
     <row r="43" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="17" t="s">
-        <v>502</v>
-      </c>
-      <c r="B43" s="17"/>
-      <c r="C43" s="17"/>
-      <c r="D43" s="17"/>
+      <c r="A43" s="18" t="s">
+        <v>529</v>
+      </c>
+      <c r="B43" s="18"/>
+      <c r="C43" s="18"/>
+      <c r="D43" s="18"/>
     </row>
     <row r="44" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="17" t="s">
-        <v>503</v>
-      </c>
-      <c r="B44" s="17"/>
-      <c r="C44" s="17"/>
-      <c r="D44" s="17"/>
+      <c r="A44" s="18" t="s">
+        <v>530</v>
+      </c>
+      <c r="B44" s="18"/>
+      <c r="C44" s="18"/>
+      <c r="D44" s="18"/>
     </row>
     <row r="45" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="17" t="s">
-        <v>504</v>
-      </c>
-      <c r="B45" s="17"/>
-      <c r="C45" s="17"/>
-      <c r="D45" s="17"/>
+      <c r="A45" s="18" t="s">
+        <v>531</v>
+      </c>
+      <c r="B45" s="18"/>
+      <c r="C45" s="18"/>
+      <c r="D45" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -7267,10 +7440,14 @@
     <mergeCell ref="A44:D44"/>
     <mergeCell ref="A45:D45"/>
   </mergeCells>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation allowBlank="false" error="Введите целое число от 0 до 10" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C6:C11" type="whole">
       <formula1>0</formula1>
       <formula2>10</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" error="Введите долю от 0 до 1 (например, 0,75)" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="B16:B19 B23:B25" type="decimal">
+      <formula1>0</formula1>
+      <formula2>1</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -7300,80 +7477,80 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>505</v>
+        <v>532</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>506</v>
+        <v>533</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>507</v>
+        <v>534</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>508</v>
+        <v>535</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>509</v>
+        <v>536</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>510</v>
+        <v>537</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>511</v>
+        <v>538</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>512</v>
+        <v>539</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>513</v>
+        <v>540</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>514</v>
+        <v>541</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>515</v>
+        <v>542</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>516</v>
+        <v>543</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>517</v>
+        <v>544</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>518</v>
+        <v>545</v>
       </c>
       <c r="E3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>519</v>
+        <v>546</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>520</v>
+        <v>547</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>521</v>
+        <v>548</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>522</v>
+        <v>549</v>
       </c>
       <c r="E4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>523</v>
+        <v>550</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>524</v>
+        <v>551</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>525</v>
+        <v>552</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>526</v>
+        <v>553</v>
       </c>
       <c r="E5" s="9"/>
     </row>
@@ -7404,170 +7581,170 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>527</v>
+        <v>554</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>528</v>
+        <v>555</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>529</v>
+        <v>556</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>530</v>
+        <v>557</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>531</v>
+        <v>558</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>532</v>
+        <v>559</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>533</v>
+        <v>560</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>534</v>
+        <v>561</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>535</v>
+        <v>562</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>536</v>
+        <v>563</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>537</v>
+        <v>564</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>538</v>
+        <v>565</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>539</v>
+        <v>566</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>540</v>
+        <v>567</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>541</v>
+        <v>568</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>542</v>
+        <v>569</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>544</v>
+        <v>571</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>545</v>
+        <v>572</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>546</v>
+        <v>573</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>547</v>
+        <v>574</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>548</v>
+        <v>575</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>549</v>
+        <v>576</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>551</v>
+        <v>578</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>552</v>
+        <v>579</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>553</v>
+        <v>580</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>554</v>
+        <v>581</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>555</v>
+        <v>582</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>556</v>
+        <v>583</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>557</v>
+        <v>584</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>558</v>
+        <v>585</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>559</v>
+        <v>586</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>560</v>
+        <v>587</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>561</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>562</v>
+        <v>589</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>563</v>
+        <v>590</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>564</v>
+        <v>591</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>565</v>
+        <v>592</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>566</v>
+        <v>593</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>567</v>
+        <v>594</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
   </sheetData>
@@ -7595,50 +7772,50 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>568</v>
+        <v>595</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>569</v>
+        <v>596</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>570</v>
+        <v>597</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>572</v>
+        <v>599</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>573</v>
+        <v>600</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>574</v>
+        <v>601</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>575</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>576</v>
+        <v>603</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>577</v>
+        <v>604</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>578</v>
+        <v>605</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>579</v>
+        <v>606</v>
       </c>
     </row>
   </sheetData>
@@ -7667,178 +7844,178 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>580</v>
+        <v>607</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>581</v>
+        <v>608</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>582</v>
+        <v>609</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>583</v>
+        <v>610</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>584</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>582</v>
+        <v>609</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>585</v>
+        <v>612</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>586</v>
+        <v>613</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="93" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>582</v>
+        <v>609</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>587</v>
+        <v>614</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>582</v>
+        <v>609</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>589</v>
+        <v>616</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>590</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>582</v>
+        <v>609</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>591</v>
+        <v>618</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>592</v>
+        <v>619</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>593</v>
+        <v>620</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>594</v>
+        <v>621</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>595</v>
+        <v>622</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>596</v>
+        <v>623</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>595</v>
+        <v>622</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>597</v>
+        <v>624</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>598</v>
+        <v>625</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>595</v>
+        <v>622</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>599</v>
+        <v>626</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>595</v>
+        <v>622</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>600</v>
+        <v>627</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="67.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>601</v>
+        <v>628</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>602</v>
+        <v>629</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>603</v>
+        <v>630</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>601</v>
+        <v>628</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>604</v>
+        <v>631</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>601</v>
+        <v>628</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>605</v>
+        <v>632</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="54.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>601</v>
+        <v>628</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>607</v>
+        <v>634</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>608</v>
+        <v>635</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>601</v>
+        <v>628</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>609</v>
+        <v>636</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>610</v>
+        <v>637</v>
       </c>
     </row>
   </sheetData>
@@ -7867,618 +8044,618 @@
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>611</v>
+        <v>638</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>612</v>
+        <v>639</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>613</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>615</v>
-      </c>
-      <c r="C2" s="18" t="s">
-        <v>616</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>642</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>617</v>
-      </c>
-      <c r="C3" s="18" t="s">
-        <v>618</v>
+        <v>644</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>645</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>619</v>
-      </c>
-      <c r="C4" s="18" t="s">
-        <v>586</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>646</v>
+      </c>
+      <c r="C4" s="19" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>620</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>621</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>647</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>622</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>623</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>649</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>624</v>
-      </c>
-      <c r="C7" s="18" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>651</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>626</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>653</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>628</v>
-      </c>
-      <c r="C9" s="18" t="s">
-        <v>629</v>
+        <v>655</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>656</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>630</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>631</v>
+        <v>657</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>658</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>632</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>610</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>659</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>633</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>634</v>
+        <v>660</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>661</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>635</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>636</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>662</v>
+      </c>
+      <c r="C13" s="19" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>637</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>606</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>664</v>
+      </c>
+      <c r="C14" s="19" t="s">
+        <v>633</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>638</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>639</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>665</v>
+      </c>
+      <c r="C15" s="19" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>640</v>
-      </c>
-      <c r="C16" s="18" t="s">
+        <v>667</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
         <v>641</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>614</v>
-      </c>
       <c r="B17" s="9" t="s">
-        <v>642</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>643</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>669</v>
+      </c>
+      <c r="C17" s="19" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>644</v>
-      </c>
-      <c r="C18" s="18" t="s">
-        <v>645</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>671</v>
+      </c>
+      <c r="C18" s="19" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>646</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>647</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>673</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>648</v>
-      </c>
-      <c r="C20" s="18" t="s">
-        <v>594</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>675</v>
+      </c>
+      <c r="C20" s="19" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>614</v>
+        <v>641</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>649</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>676</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>652</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>679</v>
+      </c>
+      <c r="C22" s="19" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>653</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>680</v>
+      </c>
+      <c r="C23" s="19" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>654</v>
-      </c>
-      <c r="C24" s="18" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>681</v>
+      </c>
+      <c r="C24" s="19" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>655</v>
-      </c>
-      <c r="C25" s="18" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>682</v>
+      </c>
+      <c r="C25" s="19" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>656</v>
-      </c>
-      <c r="C26" s="18" t="s">
-        <v>657</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>683</v>
+      </c>
+      <c r="C26" s="19" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>658</v>
-      </c>
-      <c r="C27" s="18" t="s">
-        <v>659</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>685</v>
+      </c>
+      <c r="C27" s="19" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>660</v>
-      </c>
-      <c r="C28" s="18" t="s">
-        <v>661</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>687</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>662</v>
-      </c>
-      <c r="C29" s="18" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>689</v>
+      </c>
+      <c r="C29" s="19" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>663</v>
-      </c>
-      <c r="C30" s="18" t="s">
-        <v>664</v>
+        <v>690</v>
+      </c>
+      <c r="C30" s="19" t="s">
+        <v>691</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>665</v>
-      </c>
-      <c r="C31" s="18" t="s">
-        <v>666</v>
+        <v>692</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>693</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>667</v>
-      </c>
-      <c r="C32" s="18" t="s">
-        <v>668</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>694</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>669</v>
-      </c>
-      <c r="C33" s="18" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>696</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>670</v>
-      </c>
-      <c r="C34" s="18" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>697</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>671</v>
-      </c>
-      <c r="C35" s="18" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>698</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>672</v>
-      </c>
-      <c r="C36" s="18" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>673</v>
-      </c>
-      <c r="C37" s="18" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>700</v>
+      </c>
+      <c r="C37" s="19" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>674</v>
-      </c>
-      <c r="C38" s="18" t="s">
-        <v>333</v>
+        <v>701</v>
+      </c>
+      <c r="C38" s="19" t="s">
+        <v>347</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>675</v>
-      </c>
-      <c r="C39" s="18" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>702</v>
+      </c>
+      <c r="C39" s="19" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>676</v>
-      </c>
-      <c r="C40" s="18" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>703</v>
+      </c>
+      <c r="C40" s="19" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>677</v>
-      </c>
-      <c r="C41" s="18" t="s">
-        <v>362</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>704</v>
+      </c>
+      <c r="C41" s="19" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B42" s="9" t="s">
+        <v>705</v>
+      </c>
+      <c r="C42" s="19" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="s">
         <v>678</v>
       </c>
-      <c r="C42" s="18" t="s">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="6" t="s">
-        <v>651</v>
-      </c>
       <c r="B43" s="9" t="s">
-        <v>679</v>
-      </c>
-      <c r="C43" s="18" t="s">
-        <v>376</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>706</v>
+      </c>
+      <c r="C43" s="19" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>680</v>
-      </c>
-      <c r="C44" s="18" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>707</v>
+      </c>
+      <c r="C44" s="19" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>681</v>
-      </c>
-      <c r="C45" s="18" t="s">
-        <v>399</v>
+        <v>708</v>
+      </c>
+      <c r="C45" s="19" t="s">
+        <v>418</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>682</v>
-      </c>
-      <c r="C46" s="18" t="s">
-        <v>683</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>709</v>
+      </c>
+      <c r="C46" s="19" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>684</v>
-      </c>
-      <c r="C47" s="18" t="s">
-        <v>685</v>
+        <v>711</v>
+      </c>
+      <c r="C47" s="19" t="s">
+        <v>712</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>686</v>
-      </c>
-      <c r="C48" s="18" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>713</v>
+      </c>
+      <c r="C48" s="19" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>687</v>
-      </c>
-      <c r="C49" s="18" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>714</v>
+      </c>
+      <c r="C49" s="19" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>688</v>
-      </c>
-      <c r="C50" s="18" t="s">
-        <v>438</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>715</v>
+      </c>
+      <c r="C50" s="19" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>689</v>
-      </c>
-      <c r="C51" s="18" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>716</v>
+      </c>
+      <c r="C51" s="19" t="s">
+        <v>570</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>690</v>
-      </c>
-      <c r="C52" s="18" t="s">
-        <v>691</v>
+        <v>717</v>
+      </c>
+      <c r="C52" s="19" t="s">
+        <v>718</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>692</v>
-      </c>
-      <c r="C53" s="18" t="s">
-        <v>693</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>719</v>
+      </c>
+      <c r="C53" s="19" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>694</v>
-      </c>
-      <c r="C54" s="18" t="s">
-        <v>550</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>721</v>
+      </c>
+      <c r="C54" s="19" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>695</v>
-      </c>
-      <c r="C55" s="18" t="s">
-        <v>557</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>722</v>
+      </c>
+      <c r="C55" s="19" t="s">
+        <v>584</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>651</v>
+        <v>678</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>696</v>
-      </c>
-      <c r="C56" s="18" t="s">
-        <v>561</v>
+        <v>723</v>
+      </c>
+      <c r="C56" s="19" t="s">
+        <v>588</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Polish the Excel workbook after the second verification round
- Sources use HYPERLINK formulas so long URLs wrap in LibreOffice too
- Print setup: landscape, fit to width, repeated headers; the cards
  sheet repeats the header row and ID/product columns
- Line break in the score header, wider competition/risk columns
- Capitalise the first second-tier comment
- Set document author and Russian language
- Fix the README note on MVP times for the quick-start game track

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RwfWDVGmm96bgMjE9dGnWg
</commit_message>
<xml_diff>
--- a/ideas-russia-2026.xlsx
+++ b/ideas-russia-2026.xlsx
@@ -18,7 +18,13 @@
     <sheet name="Источники" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="false" localSheetId="5" name="_xlnm.Print_Titles" vbProcedure="false">'Второй эшелон'!$1:$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="4" name="_xlnm.Print_Titles" vbProcedure="false">'Занятые ниши'!$1:$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="7" name="_xlnm.Print_Titles" vbProcedure="false">Источники!$1:$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">Карточки!$A:$B,Карточки!$1:$1</definedName>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Карточки!$A$1:$O$35</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Titles" vbProcedure="false">Кластеры!$1:$1</definedName>
+    <definedName function="false" hidden="false" localSheetId="6" name="_xlnm.Print_Titles" vbProcedure="false">'Правила рынка 2026'!$1:$1</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">Сводная!$4:$4</definedName>
     <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Сводная!$A$4:$Q$38</definedName>
   </definedNames>
@@ -150,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1168" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1113" uniqueCount="698">
   <si>
     <t xml:space="preserve">Онлайн-сервисы для России: 34 идеи, которые можно сделать с Claude Code (срез на 20.10.2026)</t>
   </si>
@@ -170,7 +176,8 @@
     <t xml:space="preserve">Тип</t>
   </si>
   <si>
-    <t xml:space="preserve">Балл (0–100)</t>
+    <t xml:space="preserve">Балл
+(0–100)</t>
   </si>
   <si>
     <t xml:space="preserve">Категория</t>
@@ -1957,7 +1964,7 @@
     <t xml:space="preserve">Профориентация с AI-симуляцией профессий</t>
   </si>
   <si>
-    <t xml:space="preserve">подросток «проживает день» хирурга, программиста или пилота. Минус: конкуренция с госпрограммами вроде «Билета в будущее».</t>
+    <t xml:space="preserve">Подросток «проживает день» хирурга, программиста или пилота. Минус: конкуренция с госпрограммами вроде «Билета в будущее».</t>
   </si>
   <si>
     <t xml:space="preserve">Детектор голосовых дипфейков для семей</t>
@@ -2099,111 +2106,63 @@
     <t xml:space="preserve">Битрикс24 — Telegram в 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.bitrix24.ru/journal/blokirovka-telegram/</t>
-  </si>
-  <si>
     <t xml:space="preserve">vc.ru — июнь 2026: Telegram, MAX, ФАС</t>
   </si>
   <si>
-    <t xml:space="preserve">https://vc.ru/telegram/2974687-blokirovka-telegram-i-ischeznoveniye-max</t>
-  </si>
-  <si>
     <t xml:space="preserve">ppc.world — WhatsApp</t>
   </si>
   <si>
     <t xml:space="preserve">Sostav — MAX для бизнеса</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.sostav.ru/blogs/292093/95285</t>
-  </si>
-  <si>
     <t xml:space="preserve">Т-Бизнес — MAX для бизнеса</t>
   </si>
   <si>
-    <t xml:space="preserve">https://secrets.tbank.ru/tehnologii/max-dlya-biznesa/</t>
-  </si>
-  <si>
     <t xml:space="preserve">Медуза — школьные чаты в Max</t>
   </si>
   <si>
-    <t xml:space="preserve">https://meduza.io/news/2025/07/27/kommersant-soobschil-chto-shkolnye-chaty-v-shesti-regionah-rossii-perevedut-v-messendzher-max-v-tatarstane-perehod-podtverdili</t>
-  </si>
-  <si>
     <t xml:space="preserve">WN Hub — Яндекс Игры, 45 млн игроков</t>
   </si>
   <si>
-    <t xml:space="preserve">https://wnhub.io/ru/news/monetization/item-47819</t>
-  </si>
-  <si>
     <t xml:space="preserve">Яндекс Игры для разработчиков</t>
   </si>
   <si>
-    <t xml:space="preserve">https://yandex.ru/project/games/for-developers</t>
-  </si>
-  <si>
     <t xml:space="preserve">ComNews — выручка игровой отрасли 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.comnews.ru/content/243534/2026-01-30/2026-w05/1008/moskva-ukrepila-liderstvo-proizvodstve-rossiyskikh-videoigr</t>
-  </si>
-  <si>
     <t xml:space="preserve">ППТ.ру — законопроект о видеоиграх</t>
   </si>
   <si>
     <t xml:space="preserve">Разбор закона об ИИ 243-ФЗ</t>
   </si>
   <si>
-    <t xml:space="preserve">https://pravo163.ru/zakon-ob-iskusstvennom-intellekte/</t>
-  </si>
-  <si>
     <t xml:space="preserve">Новая газета Европа — закон об ИИ</t>
   </si>
   <si>
-    <t xml:space="preserve">https://novayagazeta.eu/articles/2026/07/09/gosduma-priniala-pervyi-v-rossii-zakon-reguliruiushchii-rabotu-ii</t>
-  </si>
-  <si>
     <t xml:space="preserve">ППТ.ру — 289-ФЗ о платформенной экономике</t>
   </si>
   <si>
     <t xml:space="preserve">ППТ.ру — 41-ФЗ</t>
   </si>
   <si>
-    <t xml:space="preserve">https://ppt.ru/amp/obzory/vstupaet-v-silu/federalnyy-zakon-01-04-2025-41-fz</t>
-  </si>
-  <si>
     <t xml:space="preserve">Гарант — 41-ФЗ</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.garant.ru/news/1820251/</t>
-  </si>
-  <si>
     <t xml:space="preserve">3DNews — цены на модели, август 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">https://3dnews.ru/1147409</t>
-  </si>
-  <si>
     <t xml:space="preserve">AdIndex — цены на модели</t>
   </si>
   <si>
-    <t xml:space="preserve">https://adindex.ru/news/digital/2026/08/25/348304.phtml</t>
-  </si>
-  <si>
     <t xml:space="preserve">Тарифы GigaChat API</t>
   </si>
   <si>
-    <t xml:space="preserve">https://developers.sber.ru/docs/ru/gigachat/tariffs/legal-tariffs</t>
-  </si>
-  <si>
     <t xml:space="preserve">vc.ru — оплата Duolingo из РФ</t>
   </si>
   <si>
     <t xml:space="preserve">Anti-Malware — ущерб от мошенников за 2025</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.anti-malware.ru/news/2026-01-29-121598/48865</t>
-  </si>
-  <si>
     <t xml:space="preserve">Продукты и конкуренты</t>
   </si>
   <si>
@@ -2222,42 +2181,24 @@
     <t xml:space="preserve">RuStore — FoodWarz</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.rustore.ru/catalog/app/com.foodwarz.mobile</t>
-  </si>
-  <si>
     <t xml:space="preserve">Tasting Table — Timeleft</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.tastingtable.com/1859085/dinner-parties-with-strangers-timeleft</t>
-  </si>
-  <si>
     <t xml:space="preserve">Афиша — Stay Hungry</t>
   </si>
   <si>
-    <t xml:space="preserve">https://daily.afisha.ru/archive/gorod/archive/behind-stay-hungry/</t>
-  </si>
-  <si>
     <t xml:space="preserve">Storii — о StoryWorth</t>
   </si>
   <si>
     <t xml:space="preserve">Joy Calls</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.homecaremag.com/news/joy-calls-launches-ai-phone-companion-seniors</t>
-  </si>
-  <si>
     <t xml:space="preserve">Meela</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.businesswire.com/news/home/20250911525548/en/Meela-Launches-Personalized-AI-Companion-to-Combat-Loneliness-Epidemic-Among-Seniors</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rozetked — МТС и уведомления семье</t>
   </si>
   <si>
-    <t xml:space="preserve">https://rozetked.me/index.php/news/47910-analitika-bol-she-poloviny-rossiyan-ispol-zuyut-ii-servisy-cifrovoy-zaschity</t>
-  </si>
-  <si>
     <t xml:space="preserve">App Store — Laoshi AI</t>
   </si>
   <si>
@@ -2300,15 +2241,9 @@
     <t xml:space="preserve">Билайн — аудиотренажёр</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www1.ru/news/2025/04/25/ne-brat-ty-mne-audiotrenazer-ot-bilain-pomozet-otlicit-mosennika-ot-blizkogo.amp.html</t>
-  </si>
-  <si>
     <t xml:space="preserve">Product Hunt — ScamDrill</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.producthunt.com/posts/scamdrill</t>
-  </si>
-  <si>
     <t xml:space="preserve">РГ — как проверить начисления ЖКХ</t>
   </si>
   <si>
@@ -2324,13 +2259,7 @@
     <t xml:space="preserve">a2is — Скрини</t>
   </si>
   <si>
-    <t xml:space="preserve">https://a2is.ru/catalog/messendzhery-dlya-komandnoy-raboty/skrini</t>
-  </si>
-  <si>
     <t xml:space="preserve">iPhones.ru — TeamStream МТС</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.iphones.ru/iNotes/mts-web-services-otkryla-besplatnyy-dostup-k-servisu-dlya-obmena-asinhronnymi-video</t>
   </si>
   <si>
     <t xml:space="preserve">vc.ru — конструкторы свадебных сайтов</t>
@@ -3234,8 +3163,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="30"/>
   </cols>
@@ -7063,7 +6992,7 @@
   <autoFilter ref="A1:O35"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7075,7 +7004,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:D45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -7452,7 +7381,7 @@
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7463,7 +7392,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -7557,7 +7486,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7568,7 +7497,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:D12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -7750,7 +7679,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7761,7 +7690,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:B6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -7821,7 +7750,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7832,7 +7761,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -8021,7 +7950,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -8032,7 +7961,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C56"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -8060,8 +7989,9 @@
       <c r="B2" s="9" t="s">
         <v>642</v>
       </c>
-      <c r="C2" s="19" t="s">
-        <v>643</v>
+      <c r="C2" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.bitrix24.ru/journal/blokirovka-telegram/","https://www.bitrix24.ru/journal/blokirovka-telegram/")</f>
+        <v>https://www.bitrix24.ru/journal/blokirovka-telegram/</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8069,10 +7999,11 @@
         <v>641</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>644</v>
-      </c>
-      <c r="C3" s="19" t="s">
-        <v>645</v>
+        <v>643</v>
+      </c>
+      <c r="C3" s="19" t="str">
+        <f aca="false">HYPERLINK("https://vc.ru/telegram/2974687-blokirovka-telegram-i-ischeznoveniye-max","https://vc.ru/telegram/2974687-blokirovka-telegram-i-ischeznoveniye-max")</f>
+        <v>https://vc.ru/telegram/2974687-blokirovka-telegram-i-ischeznoveniye-max</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8080,10 +8011,11 @@
         <v>641</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>646</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>613</v>
+        <v>644</v>
+      </c>
+      <c r="C4" s="19" t="str">
+        <f aca="false">HYPERLINK("https://ppc.world/news/whatsapp-otklyuchat-v-2026-godu-telegram-trogat-ne-budut-deputat-gosdumy/","https://ppc.world/news/whatsapp-otklyuchat-v-2026-godu-telegram-trogat-ne-budut-deputat-gosdumy/")</f>
+        <v>https://ppc.world/news/whatsapp-otklyuchat-v-2026-godu-telegram-trogat-ne-budut-deputat-gosdumy/</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8091,10 +8023,11 @@
         <v>641</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>647</v>
-      </c>
-      <c r="C5" s="19" t="s">
-        <v>648</v>
+        <v>645</v>
+      </c>
+      <c r="C5" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.sostav.ru/blogs/292093/95285","https://www.sostav.ru/blogs/292093/95285")</f>
+        <v>https://www.sostav.ru/blogs/292093/95285</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8102,10 +8035,11 @@
         <v>641</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>649</v>
-      </c>
-      <c r="C6" s="19" t="s">
-        <v>650</v>
+        <v>646</v>
+      </c>
+      <c r="C6" s="19" t="str">
+        <f aca="false">HYPERLINK("https://secrets.tbank.ru/tehnologii/max-dlya-biznesa/","https://secrets.tbank.ru/tehnologii/max-dlya-biznesa/")</f>
+        <v>https://secrets.tbank.ru/tehnologii/max-dlya-biznesa/</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8113,10 +8047,11 @@
         <v>641</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>651</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>652</v>
+        <v>647</v>
+      </c>
+      <c r="C7" s="19" t="str">
+        <f aca="false">HYPERLINK("https://meduza.io/news/2025/07/27/kommersant-soobschil-chto-shkolnye-chaty-v-shesti-regionah-rossii-perevedut-v-messendzher-max-v-tatarstane-perehod-podtverdili","https://meduza.io/news/2025/07/27/kommersant-soobschil-chto-shkolnye-chaty-v-shesti-regionah-rossii-perevedut-v-messendzher-max-v-tatarstane-perehod-podtverdili")</f>
+        <v>https://meduza.io/news/2025/07/27/kommersant-soobschil-chto-shkolnye-chaty-v-shesti-regionah-rossii-perevedut-v-messendzher-max-v-tatarstane-perehod-podtverdili</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8124,10 +8059,11 @@
         <v>641</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>653</v>
-      </c>
-      <c r="C8" s="19" t="s">
-        <v>654</v>
+        <v>648</v>
+      </c>
+      <c r="C8" s="19" t="str">
+        <f aca="false">HYPERLINK("https://wnhub.io/ru/news/monetization/item-47819","https://wnhub.io/ru/news/monetization/item-47819")</f>
+        <v>https://wnhub.io/ru/news/monetization/item-47819</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8135,10 +8071,11 @@
         <v>641</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>655</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>656</v>
+        <v>649</v>
+      </c>
+      <c r="C9" s="19" t="str">
+        <f aca="false">HYPERLINK("https://yandex.ru/project/games/for-developers","https://yandex.ru/project/games/for-developers")</f>
+        <v>https://yandex.ru/project/games/for-developers</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8146,10 +8083,11 @@
         <v>641</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>657</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>658</v>
+        <v>650</v>
+      </c>
+      <c r="C10" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.comnews.ru/content/243534/2026-01-30/2026-w05/1008/moskva-ukrepila-liderstvo-proizvodstve-rossiyskikh-videoigr","https://www.comnews.ru/content/243534/2026-01-30/2026-w05/1008/moskva-ukrepila-liderstvo-proizvodstve-rossiyskikh-videoigr")</f>
+        <v>https://www.comnews.ru/content/243534/2026-01-30/2026-w05/1008/moskva-ukrepila-liderstvo-proizvodstve-rossiyskikh-videoigr</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8157,10 +8095,11 @@
         <v>641</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>659</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>637</v>
+        <v>651</v>
+      </c>
+      <c r="C11" s="19" t="str">
+        <f aca="false">HYPERLINK("https://ppt.ru/news/identifikatsiya-klientov/vvedut-markirovku-i-identifikatsiyu-igrokov-v-videoigrakh","https://ppt.ru/news/identifikatsiya-klientov/vvedut-markirovku-i-identifikatsiyu-igrokov-v-videoigrakh")</f>
+        <v>https://ppt.ru/news/identifikatsiya-klientov/vvedut-markirovku-i-identifikatsiyu-igrokov-v-videoigrakh</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8168,10 +8107,11 @@
         <v>641</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>660</v>
-      </c>
-      <c r="C12" s="19" t="s">
-        <v>661</v>
+        <v>652</v>
+      </c>
+      <c r="C12" s="19" t="str">
+        <f aca="false">HYPERLINK("https://pravo163.ru/zakon-ob-iskusstvennom-intellekte/","https://pravo163.ru/zakon-ob-iskusstvennom-intellekte/")</f>
+        <v>https://pravo163.ru/zakon-ob-iskusstvennom-intellekte/</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8179,10 +8119,11 @@
         <v>641</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>662</v>
-      </c>
-      <c r="C13" s="19" t="s">
-        <v>663</v>
+        <v>653</v>
+      </c>
+      <c r="C13" s="19" t="str">
+        <f aca="false">HYPERLINK("https://novayagazeta.eu/articles/2026/07/09/gosduma-priniala-pervyi-v-rossii-zakon-reguliruiushchii-rabotu-ii","https://novayagazeta.eu/articles/2026/07/09/gosduma-priniala-pervyi-v-rossii-zakon-reguliruiushchii-rabotu-ii")</f>
+        <v>https://novayagazeta.eu/articles/2026/07/09/gosduma-priniala-pervyi-v-rossii-zakon-reguliruiushchii-rabotu-ii</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8190,10 +8131,11 @@
         <v>641</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>664</v>
-      </c>
-      <c r="C14" s="19" t="s">
-        <v>633</v>
+        <v>654</v>
+      </c>
+      <c r="C14" s="19" t="str">
+        <f aca="false">HYPERLINK("https://ppt.ru/obzory/vstupaet-v-silu/federalnyy-zakon-31-07-2025-289-fz","https://ppt.ru/obzory/vstupaet-v-silu/federalnyy-zakon-31-07-2025-289-fz")</f>
+        <v>https://ppt.ru/obzory/vstupaet-v-silu/federalnyy-zakon-31-07-2025-289-fz</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8201,10 +8143,11 @@
         <v>641</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>665</v>
-      </c>
-      <c r="C15" s="19" t="s">
-        <v>666</v>
+        <v>655</v>
+      </c>
+      <c r="C15" s="19" t="str">
+        <f aca="false">HYPERLINK("https://ppt.ru/amp/obzory/vstupaet-v-silu/federalnyy-zakon-01-04-2025-41-fz","https://ppt.ru/amp/obzory/vstupaet-v-silu/federalnyy-zakon-01-04-2025-41-fz")</f>
+        <v>https://ppt.ru/amp/obzory/vstupaet-v-silu/federalnyy-zakon-01-04-2025-41-fz</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8212,10 +8155,11 @@
         <v>641</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>667</v>
-      </c>
-      <c r="C16" s="19" t="s">
-        <v>668</v>
+        <v>656</v>
+      </c>
+      <c r="C16" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.garant.ru/news/1820251/","https://www.garant.ru/news/1820251/")</f>
+        <v>https://www.garant.ru/news/1820251/</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8223,10 +8167,11 @@
         <v>641</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>669</v>
-      </c>
-      <c r="C17" s="19" t="s">
-        <v>670</v>
+        <v>657</v>
+      </c>
+      <c r="C17" s="19" t="str">
+        <f aca="false">HYPERLINK("https://3dnews.ru/1147409","https://3dnews.ru/1147409")</f>
+        <v>https://3dnews.ru/1147409</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8234,10 +8179,11 @@
         <v>641</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>671</v>
-      </c>
-      <c r="C18" s="19" t="s">
-        <v>672</v>
+        <v>658</v>
+      </c>
+      <c r="C18" s="19" t="str">
+        <f aca="false">HYPERLINK("https://adindex.ru/news/digital/2026/08/25/348304.phtml","https://adindex.ru/news/digital/2026/08/25/348304.phtml")</f>
+        <v>https://adindex.ru/news/digital/2026/08/25/348304.phtml</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8245,10 +8191,11 @@
         <v>641</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>673</v>
-      </c>
-      <c r="C19" s="19" t="s">
-        <v>674</v>
+        <v>659</v>
+      </c>
+      <c r="C19" s="19" t="str">
+        <f aca="false">HYPERLINK("https://developers.sber.ru/docs/ru/gigachat/tariffs/legal-tariffs","https://developers.sber.ru/docs/ru/gigachat/tariffs/legal-tariffs")</f>
+        <v>https://developers.sber.ru/docs/ru/gigachat/tariffs/legal-tariffs</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8256,10 +8203,11 @@
         <v>641</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>675</v>
-      </c>
-      <c r="C20" s="19" t="s">
-        <v>621</v>
+        <v>660</v>
+      </c>
+      <c r="C20" s="19" t="str">
+        <f aca="false">HYPERLINK("https://vc.ru/services/3012698-sposoby-oplaty-podpiski-duolingo-iz-rossii","https://vc.ru/services/3012698-sposoby-oplaty-podpiski-duolingo-iz-rossii")</f>
+        <v>https://vc.ru/services/3012698-sposoby-oplaty-podpiski-duolingo-iz-rossii</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8267,458 +8215,437 @@
         <v>641</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>676</v>
-      </c>
-      <c r="C21" s="19" t="s">
-        <v>677</v>
+        <v>661</v>
+      </c>
+      <c r="C21" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.anti-malware.ru/news/2026-01-29-121598/48865","https://www.anti-malware.ru/news/2026-01-29-121598/48865")</f>
+        <v>https://www.anti-malware.ru/news/2026-01-29-121598/48865</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>679</v>
-      </c>
-      <c r="C22" s="19" t="s">
-        <v>219</v>
+        <v>663</v>
+      </c>
+      <c r="C22" s="19" t="str">
+        <f aca="false">HYPERLINK("https://t-j.ru/5bukv-game-stat/","https://t-j.ru/5bukv-game-stat/")</f>
+        <v>https://t-j.ru/5bukv-game-stat/</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>680</v>
-      </c>
-      <c r="C23" s="19" t="s">
-        <v>227</v>
+        <v>664</v>
+      </c>
+      <c r="C23" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.jackboxgames.com/how-to","https://www.jackboxgames.com/how-to")</f>
+        <v>https://www.jackboxgames.com/how-to</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>681</v>
-      </c>
-      <c r="C24" s="19" t="s">
-        <v>244</v>
+        <v>665</v>
+      </c>
+      <c r="C24" s="19" t="str">
+        <f aca="false">HYPERLINK("https://naked-science.ru/article/media/onlaine-game-geoguessr","https://naked-science.ru/article/media/onlaine-game-geoguessr")</f>
+        <v>https://naked-science.ru/article/media/onlaine-game-geoguessr</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>682</v>
-      </c>
-      <c r="C25" s="19" t="s">
-        <v>261</v>
+        <v>666</v>
+      </c>
+      <c r="C25" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.rustore.ru/catalog/app/com.nutrisync.advanced","https://www.rustore.ru/catalog/app/com.nutrisync.advanced")</f>
+        <v>https://www.rustore.ru/catalog/app/com.nutrisync.advanced</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>683</v>
-      </c>
-      <c r="C26" s="19" t="s">
-        <v>684</v>
+        <v>667</v>
+      </c>
+      <c r="C26" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.rustore.ru/catalog/app/com.foodwarz.mobile","https://www.rustore.ru/catalog/app/com.foodwarz.mobile")</f>
+        <v>https://www.rustore.ru/catalog/app/com.foodwarz.mobile</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>685</v>
-      </c>
-      <c r="C27" s="19" t="s">
-        <v>686</v>
+        <v>668</v>
+      </c>
+      <c r="C27" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.tastingtable.com/1859085/dinner-parties-with-strangers-timeleft","https://www.tastingtable.com/1859085/dinner-parties-with-strangers-timeleft")</f>
+        <v>https://www.tastingtable.com/1859085/dinner-parties-with-strangers-timeleft</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>687</v>
-      </c>
-      <c r="C28" s="19" t="s">
-        <v>688</v>
+        <v>669</v>
+      </c>
+      <c r="C28" s="19" t="str">
+        <f aca="false">HYPERLINK("https://daily.afisha.ru/archive/gorod/archive/behind-stay-hungry/","https://daily.afisha.ru/archive/gorod/archive/behind-stay-hungry/")</f>
+        <v>https://daily.afisha.ru/archive/gorod/archive/behind-stay-hungry/</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>689</v>
-      </c>
-      <c r="C29" s="19" t="s">
-        <v>279</v>
+        <v>670</v>
+      </c>
+      <c r="C29" s="19" t="str">
+        <f aca="false">HYPERLINK("https://storii.com/blog/storyworth","https://storii.com/blog/storyworth")</f>
+        <v>https://storii.com/blog/storyworth</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>690</v>
-      </c>
-      <c r="C30" s="19" t="s">
-        <v>691</v>
+        <v>671</v>
+      </c>
+      <c r="C30" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.homecaremag.com/news/joy-calls-launches-ai-phone-companion-seniors","https://www.homecaremag.com/news/joy-calls-launches-ai-phone-companion-seniors")</f>
+        <v>https://www.homecaremag.com/news/joy-calls-launches-ai-phone-companion-seniors</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>692</v>
-      </c>
-      <c r="C31" s="19" t="s">
-        <v>693</v>
+        <v>672</v>
+      </c>
+      <c r="C31" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.businesswire.com/news/home/20250911525548/en/Meela-Launches-Personalized-AI-Companion-to-Combat-Loneliness-Epidemic-Among-Seniors","https://www.businesswire.com/news/home/20250911525548/en/Meela-Launches-Personalized-AI-Companion-to-Combat-Loneliness-Epidemic-Among-Seniors")</f>
+        <v>https://www.businesswire.com/news/home/20250911525548/en/Meela-Launches-Personalized-AI-Companion-to-Combat-Loneliness-Epidemic-Among-Seniors</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>694</v>
-      </c>
-      <c r="C32" s="19" t="s">
-        <v>695</v>
+        <v>673</v>
+      </c>
+      <c r="C32" s="19" t="str">
+        <f aca="false">HYPERLINK("https://rozetked.me/index.php/news/47910-analitika-bol-she-poloviny-rossiyan-ispol-zuyut-ii-servisy-cifrovoy-zaschity","https://rozetked.me/index.php/news/47910-analitika-bol-she-poloviny-rossiyan-ispol-zuyut-ii-servisy-cifrovoy-zaschity")</f>
+        <v>https://rozetked.me/index.php/news/47910-analitika-bol-she-poloviny-rossiyan-ispol-zuyut-ii-servisy-cifrovoy-zaschity</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>696</v>
-      </c>
-      <c r="C33" s="19" t="s">
-        <v>297</v>
+        <v>674</v>
+      </c>
+      <c r="C33" s="19" t="str">
+        <f aca="false">HYPERLINK("https://apps.apple.com/us/app/%D0%BA%D0%B8%D1%82%D0%B0%D0%B9%D1%81%D0%BA%D0%B8%D0%B9-%D1%8F%D0%B7%D1%8B%D0%BA-%D1%81-%D0%BB%D0%B0%D0%BE%D1%88%D0%B8/id1510215770?l=ru","https://apps.apple.com/us/app/%D0%BA%D0%B8%D1%82%D0%B0%D0%B9%D1%81%D0%BA%D0%B8%D0%B9-%D1%8F%D0%B7%D1%8B%D0%BA-%D1%81-%D0%BB%D0%B0%D0%BE%D1%88%D0%B8/id1510215770?l=ru")</f>
+        <v>https://apps.apple.com/us/app/%D0%BA%D0%B8%D1%82%D0%B0%D0%B9%D1%81%D0%BA%D0%B8%D0%B9-%D1%8F%D0%B7%D1%8B%D0%BA-%D1%81-%D0%BB%D0%B0%D0%BE%D1%88%D0%B8/id1510215770?l=ru</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>697</v>
-      </c>
-      <c r="C34" s="19" t="s">
-        <v>314</v>
+        <v>675</v>
+      </c>
+      <c r="C34" s="19" t="str">
+        <f aca="false">HYPERLINK("https://yandex.cloud/ru/cases/aipushkin","https://yandex.cloud/ru/cases/aipushkin")</f>
+        <v>https://yandex.cloud/ru/cases/aipushkin</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>698</v>
-      </c>
-      <c r="C35" s="19" t="s">
-        <v>322</v>
+        <v>676</v>
+      </c>
+      <c r="C35" s="19" t="str">
+        <f aca="false">HYPERLINK("https://developers.sber.ru/help/gigachat-api/ai-for-teachers","https://developers.sber.ru/help/gigachat-api/ai-for-teachers")</f>
+        <v>https://developers.sber.ru/help/gigachat-api/ai-for-teachers</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>699</v>
-      </c>
-      <c r="C36" s="19" t="s">
-        <v>331</v>
+        <v>677</v>
+      </c>
+      <c r="C36" s="19" t="str">
+        <f aca="false">HYPERLINK("https://apps.apple.com/ru/app/id6471586789","https://apps.apple.com/ru/app/id6471586789")</f>
+        <v>https://apps.apple.com/ru/app/id6471586789</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
+        <v>662</v>
+      </c>
+      <c r="B37" s="9" t="s">
         <v>678</v>
       </c>
-      <c r="B37" s="9" t="s">
-        <v>700</v>
-      </c>
-      <c r="C37" s="19" t="s">
-        <v>339</v>
+      <c r="C37" s="19" t="str">
+        <f aca="false">HYPERLINK("https://pravoved.ru/documents/new/claim/","https://pravoved.ru/documents/new/claim/")</f>
+        <v>https://pravoved.ru/documents/new/claim/</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>701</v>
-      </c>
-      <c r="C38" s="19" t="s">
-        <v>347</v>
+        <v>679</v>
+      </c>
+      <c r="C38" s="19" t="str">
+        <f aca="false">HYPERLINK("https://vitvet.com/articles/bankrotstvo/vnesudebnoe_bankrotstvo_mfc/","https://vitvet.com/articles/bankrotstvo/vnesudebnoe_bankrotstvo_mfc/")</f>
+        <v>https://vitvet.com/articles/bankrotstvo/vnesudebnoe_bankrotstvo_mfc/</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>702</v>
-      </c>
-      <c r="C39" s="19" t="s">
-        <v>355</v>
+        <v>680</v>
+      </c>
+      <c r="C39" s="19" t="str">
+        <f aca="false">HYPERLINK("https://finuslugi.ru/navigator/kak-ehto-rabotaet/stat_semeynaya-nalogovaya-vyplata-v-2026-godu","https://finuslugi.ru/navigator/kak-ehto-rabotaet/stat_semeynaya-nalogovaya-vyplata-v-2026-godu")</f>
+        <v>https://finuslugi.ru/navigator/kak-ehto-rabotaet/stat_semeynaya-nalogovaya-vyplata-v-2026-godu</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>703</v>
-      </c>
-      <c r="C40" s="19" t="s">
-        <v>364</v>
+        <v>681</v>
+      </c>
+      <c r="C40" s="19" t="str">
+        <f aca="false">HYPERLINK("https://workspace.ru/cases/puteshestviya-po-rossii-ot-neyroseti/","https://workspace.ru/cases/puteshestviya-po-rossii-ot-neyroseti/")</f>
+        <v>https://workspace.ru/cases/puteshestviya-po-rossii-ot-neyroseti/</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>704</v>
-      </c>
-      <c r="C41" s="19" t="s">
-        <v>379</v>
+        <v>682</v>
+      </c>
+      <c r="C41" s="19" t="str">
+        <f aca="false">HYPERLINK("https://t-j.ru/smogut-li-prizhitsia-v-rossii-servisy-po-spaseniiu-edy/","https://t-j.ru/smogut-li-prizhitsia-v-rossii-servisy-po-spaseniiu-edy/")</f>
+        <v>https://t-j.ru/smogut-li-prizhitsia-v-rossii-servisy-po-spaseniiu-edy/</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>705</v>
-      </c>
-      <c r="C42" s="19" t="s">
-        <v>386</v>
+        <v>683</v>
+      </c>
+      <c r="C42" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.rustore.ru/catalog/app/ru.dacha.app","https://www.rustore.ru/catalog/app/ru.dacha.app")</f>
+        <v>https://www.rustore.ru/catalog/app/ru.dacha.app</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>706</v>
-      </c>
-      <c r="C43" s="19" t="s">
-        <v>394</v>
+        <v>684</v>
+      </c>
+      <c r="C43" s="19" t="str">
+        <f aca="false">HYPERLINK("https://t-j.ru/discount-aggregators/","https://t-j.ru/discount-aggregators/")</f>
+        <v>https://t-j.ru/discount-aggregators/</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>707</v>
-      </c>
-      <c r="C44" s="19" t="s">
-        <v>403</v>
+        <v>685</v>
+      </c>
+      <c r="C44" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.stork.ai/collections/ru/ai-receptionists-salon","https://www.stork.ai/collections/ru/ai-receptionists-salon")</f>
+        <v>https://www.stork.ai/collections/ru/ai-receptionists-salon</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>708</v>
-      </c>
-      <c r="C45" s="19" t="s">
-        <v>418</v>
+        <v>686</v>
+      </c>
+      <c r="C45" s="19" t="str">
+        <f aca="false">HYPERLINK("https://lifehacker.ru/yousician-guitar/","https://lifehacker.ru/yousician-guitar/")</f>
+        <v>https://lifehacker.ru/yousician-guitar/</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>709</v>
-      </c>
-      <c r="C46" s="19" t="s">
-        <v>710</v>
+        <v>687</v>
+      </c>
+      <c r="C46" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www1.ru/news/2025/04/25/ne-brat-ty-mne-audiotrenazer-ot-bilain-pomozet-otlicit-mosennika-ot-blizkogo.amp.html","https://www1.ru/news/2025/04/25/ne-brat-ty-mne-audiotrenazer-ot-bilain-pomozet-otlicit-mosennika-ot-blizkogo.amp.html")</f>
+        <v>https://www1.ru/news/2025/04/25/ne-brat-ty-mne-audiotrenazer-ot-bilain-pomozet-otlicit-mosennika-ot-blizkogo.amp.html</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>711</v>
-      </c>
-      <c r="C47" s="19" t="s">
-        <v>712</v>
+        <v>688</v>
+      </c>
+      <c r="C47" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.producthunt.com/posts/scamdrill","https://www.producthunt.com/posts/scamdrill")</f>
+        <v>https://www.producthunt.com/posts/scamdrill</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>713</v>
-      </c>
-      <c r="C48" s="19" t="s">
-        <v>435</v>
+        <v>689</v>
+      </c>
+      <c r="C48" s="19" t="str">
+        <f aca="false">HYPERLINK("https://rg.ru/post/kak-proverit-nachisleniia-za-kommunalnye-uslugi-i-ne-pereplatit-za-zhkh.html","https://rg.ru/post/kak-proverit-nachisleniia-za-kommunalnye-uslugi-i-ne-pereplatit-za-zhkh.html")</f>
+        <v>https://rg.ru/post/kak-proverit-nachisleniia-za-kommunalnye-uslugi-i-ne-pereplatit-za-zhkh.html</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>714</v>
-      </c>
-      <c r="C49" s="19" t="s">
-        <v>444</v>
+        <v>690</v>
+      </c>
+      <c r="C49" s="19" t="str">
+        <f aca="false">HYPERLINK("https://spark.ru/startup/vs-na-strojku/blog/350477/sdelal-servis-kotorij-proveryaet-smeti-na-remont-za-pervuyu-nedelyu-nashli-pereplat-na-1-5-milliona-rublej","https://spark.ru/startup/vs-na-strojku/blog/350477/sdelal-servis-kotorij-proveryaet-smeti-na-remont-za-pervuyu-nedelyu-nashli-pereplat-na-1-5-milliona-rublej")</f>
+        <v>https://spark.ru/startup/vs-na-strojku/blog/350477/sdelal-servis-kotorij-proveryaet-smeti-na-remont-za-pervuyu-nedelyu-nashli-pereplat-na-1-5-milliona-rublej</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>715</v>
-      </c>
-      <c r="C50" s="19" t="s">
-        <v>461</v>
+        <v>691</v>
+      </c>
+      <c r="C50" s="19" t="str">
+        <f aca="false">HYPERLINK("https://dtf.ru/indie/5178362-rezhim-zhivye-podozrevaemye-v-case-zero","https://dtf.ru/indie/5178362-rezhim-zhivye-podozrevaemye-v-case-zero")</f>
+        <v>https://dtf.ru/indie/5178362-rezhim-zhivye-podozrevaemye-v-case-zero</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>716</v>
-      </c>
-      <c r="C51" s="19" t="s">
-        <v>570</v>
+        <v>692</v>
+      </c>
+      <c r="C51" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.sostav.ru/blogs/290467/88610","https://www.sostav.ru/blogs/290467/88610")</f>
+        <v>https://www.sostav.ru/blogs/290467/88610</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>717</v>
-      </c>
-      <c r="C52" s="19" t="s">
-        <v>718</v>
+        <v>693</v>
+      </c>
+      <c r="C52" s="19" t="str">
+        <f aca="false">HYPERLINK("https://a2is.ru/catalog/messendzhery-dlya-komandnoy-raboty/skrini","https://a2is.ru/catalog/messendzhery-dlya-komandnoy-raboty/skrini")</f>
+        <v>https://a2is.ru/catalog/messendzhery-dlya-komandnoy-raboty/skrini</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B53" s="9" t="s">
-        <v>719</v>
-      </c>
-      <c r="C53" s="19" t="s">
-        <v>720</v>
+        <v>694</v>
+      </c>
+      <c r="C53" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.iphones.ru/iNotes/mts-web-services-otkryla-besplatnyy-dostup-k-servisu-dlya-obmena-asinhronnymi-video","https://www.iphones.ru/iNotes/mts-web-services-otkryla-besplatnyy-dostup-k-servisu-dlya-obmena-asinhronnymi-video")</f>
+        <v>https://www.iphones.ru/iNotes/mts-web-services-otkryla-besplatnyy-dostup-k-servisu-dlya-obmena-asinhronnymi-video</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>721</v>
-      </c>
-      <c r="C54" s="19" t="s">
-        <v>577</v>
+        <v>695</v>
+      </c>
+      <c r="C54" s="19" t="str">
+        <f aca="false">HYPERLINK("https://vc.ru/services/3041069-konstruktor-saytov-svadb-privlecheniy","https://vc.ru/services/3041069-konstruktor-saytov-svadb-privlecheniy")</f>
+        <v>https://vc.ru/services/3041069-konstruktor-saytov-svadb-privlecheniy</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>722</v>
-      </c>
-      <c r="C55" s="19" t="s">
-        <v>584</v>
+        <v>696</v>
+      </c>
+      <c r="C55" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.rustore.ru/catalog/app/ru.komod.app","https://www.rustore.ru/catalog/app/ru.komod.app")</f>
+        <v>https://www.rustore.ru/catalog/app/ru.komod.app</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="6" t="s">
-        <v>678</v>
+        <v>662</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>723</v>
-      </c>
-      <c r="C56" s="19" t="s">
-        <v>588</v>
+        <v>697</v>
+      </c>
+      <c r="C56" s="19" t="str">
+        <f aca="false">HYPERLINK("https://www.rustore.ru/catalog/app/click.opora.app","https://www.rustore.ru/catalog/app/click.opora.app")</f>
+        <v>https://www.rustore.ru/catalog/app/click.opora.app</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" display="https://www.bitrix24.ru/journal/blokirovka-telegram/"/>
-    <hyperlink ref="C3" r:id="rId2" display="https://vc.ru/telegram/2974687-blokirovka-telegram-i-ischeznoveniye-max"/>
-    <hyperlink ref="C4" r:id="rId3" display="https://ppc.world/news/whatsapp-otklyuchat-v-2026-godu-telegram-trogat-ne-budut-deputat-gosdumy/"/>
-    <hyperlink ref="C5" r:id="rId4" display="https://www.sostav.ru/blogs/292093/95285"/>
-    <hyperlink ref="C6" r:id="rId5" display="https://secrets.tbank.ru/tehnologii/max-dlya-biznesa/"/>
-    <hyperlink ref="C7" r:id="rId6" display="https://meduza.io/news/2025/07/27/kommersant-soobschil-chto-shkolnye-chaty-v-shesti-regionah-rossii-perevedut-v-messendzher-max-v-tatarstane-perehod-podtverdili"/>
-    <hyperlink ref="C8" r:id="rId7" display="https://wnhub.io/ru/news/monetization/item-47819"/>
-    <hyperlink ref="C9" r:id="rId8" display="https://yandex.ru/project/games/for-developers"/>
-    <hyperlink ref="C10" r:id="rId9" display="https://www.comnews.ru/content/243534/2026-01-30/2026-w05/1008/moskva-ukrepila-liderstvo-proizvodstve-rossiyskikh-videoigr"/>
-    <hyperlink ref="C11" r:id="rId10" display="https://ppt.ru/news/identifikatsiya-klientov/vvedut-markirovku-i-identifikatsiyu-igrokov-v-videoigrakh"/>
-    <hyperlink ref="C12" r:id="rId11" display="https://pravo163.ru/zakon-ob-iskusstvennom-intellekte/"/>
-    <hyperlink ref="C13" r:id="rId12" display="https://novayagazeta.eu/articles/2026/07/09/gosduma-priniala-pervyi-v-rossii-zakon-reguliruiushchii-rabotu-ii"/>
-    <hyperlink ref="C14" r:id="rId13" display="https://ppt.ru/obzory/vstupaet-v-silu/federalnyy-zakon-31-07-2025-289-fz"/>
-    <hyperlink ref="C15" r:id="rId14" display="https://ppt.ru/amp/obzory/vstupaet-v-silu/federalnyy-zakon-01-04-2025-41-fz"/>
-    <hyperlink ref="C16" r:id="rId15" display="https://www.garant.ru/news/1820251/"/>
-    <hyperlink ref="C17" r:id="rId16" display="https://3dnews.ru/1147409"/>
-    <hyperlink ref="C18" r:id="rId17" display="https://adindex.ru/news/digital/2026/08/25/348304.phtml"/>
-    <hyperlink ref="C19" r:id="rId18" display="https://developers.sber.ru/docs/ru/gigachat/tariffs/legal-tariffs"/>
-    <hyperlink ref="C20" r:id="rId19" display="https://vc.ru/services/3012698-sposoby-oplaty-podpiski-duolingo-iz-rossii"/>
-    <hyperlink ref="C21" r:id="rId20" display="https://www.anti-malware.ru/news/2026-01-29-121598/48865"/>
-    <hyperlink ref="C22" r:id="rId21" display="https://t-j.ru/5bukv-game-stat/"/>
-    <hyperlink ref="C23" r:id="rId22" display="https://www.jackboxgames.com/how-to"/>
-    <hyperlink ref="C24" r:id="rId23" display="https://naked-science.ru/article/media/onlaine-game-geoguessr"/>
-    <hyperlink ref="C25" r:id="rId24" display="https://www.rustore.ru/catalog/app/com.nutrisync.advanced"/>
-    <hyperlink ref="C26" r:id="rId25" display="https://www.rustore.ru/catalog/app/com.foodwarz.mobile"/>
-    <hyperlink ref="C27" r:id="rId26" display="https://www.tastingtable.com/1859085/dinner-parties-with-strangers-timeleft"/>
-    <hyperlink ref="C28" r:id="rId27" display="https://daily.afisha.ru/archive/gorod/archive/behind-stay-hungry/"/>
-    <hyperlink ref="C29" r:id="rId28" display="https://storii.com/blog/storyworth"/>
-    <hyperlink ref="C30" r:id="rId29" display="https://www.homecaremag.com/news/joy-calls-launches-ai-phone-companion-seniors"/>
-    <hyperlink ref="C31" r:id="rId30" display="https://www.businesswire.com/news/home/20250911525548/en/Meela-Launches-Personalized-AI-Companion-to-Combat-Loneliness-Epidemic-Among-Seniors"/>
-    <hyperlink ref="C32" r:id="rId31" display="https://rozetked.me/index.php/news/47910-analitika-bol-she-poloviny-rossiyan-ispol-zuyut-ii-servisy-cifrovoy-zaschity"/>
-    <hyperlink ref="C33" r:id="rId32" display="https://apps.apple.com/us/app/%D0%BA%D0%B8%D1%82%D0%B0%D0%B9%D1%81%D0%BA%D0%B8%D0%B9-%D1%8F%D0%B7%D1%8B%D0%BA-%D1%81-%D0%BB%D0%B0%D0%BE%D1%88%D0%B8/id1510215770?l=ru"/>
-    <hyperlink ref="C34" r:id="rId33" display="https://yandex.cloud/ru/cases/aipushkin"/>
-    <hyperlink ref="C35" r:id="rId34" display="https://developers.sber.ru/help/gigachat-api/ai-for-teachers"/>
-    <hyperlink ref="C36" r:id="rId35" display="https://apps.apple.com/ru/app/id6471586789"/>
-    <hyperlink ref="C37" r:id="rId36" display="https://pravoved.ru/documents/new/claim/"/>
-    <hyperlink ref="C38" r:id="rId37" display="https://vitvet.com/articles/bankrotstvo/vnesudebnoe_bankrotstvo_mfc/"/>
-    <hyperlink ref="C39" r:id="rId38" display="https://finuslugi.ru/navigator/kak-ehto-rabotaet/stat_semeynaya-nalogovaya-vyplata-v-2026-godu"/>
-    <hyperlink ref="C40" r:id="rId39" display="https://workspace.ru/cases/puteshestviya-po-rossii-ot-neyroseti/"/>
-    <hyperlink ref="C41" r:id="rId40" display="https://t-j.ru/smogut-li-prizhitsia-v-rossii-servisy-po-spaseniiu-edy/"/>
-    <hyperlink ref="C42" r:id="rId41" display="https://www.rustore.ru/catalog/app/ru.dacha.app"/>
-    <hyperlink ref="C43" r:id="rId42" display="https://t-j.ru/discount-aggregators/"/>
-    <hyperlink ref="C44" r:id="rId43" display="https://www.stork.ai/collections/ru/ai-receptionists-salon"/>
-    <hyperlink ref="C45" r:id="rId44" display="https://lifehacker.ru/yousician-guitar/"/>
-    <hyperlink ref="C46" r:id="rId45" display="https://www1.ru/news/2025/04/25/ne-brat-ty-mne-audiotrenazer-ot-bilain-pomozet-otlicit-mosennika-ot-blizkogo.amp.html"/>
-    <hyperlink ref="C47" r:id="rId46" display="https://www.producthunt.com/posts/scamdrill"/>
-    <hyperlink ref="C48" r:id="rId47" display="https://rg.ru/post/kak-proverit-nachisleniia-za-kommunalnye-uslugi-i-ne-pereplatit-za-zhkh.html"/>
-    <hyperlink ref="C49" r:id="rId48" display="https://spark.ru/startup/vs-na-strojku/blog/350477/sdelal-servis-kotorij-proveryaet-smeti-na-remont-za-pervuyu-nedelyu-nashli-pereplat-na-1-5-milliona-rublej"/>
-    <hyperlink ref="C50" r:id="rId49" display="https://dtf.ru/indie/5178362-rezhim-zhivye-podozrevaemye-v-case-zero"/>
-    <hyperlink ref="C51" r:id="rId50" display="https://www.sostav.ru/blogs/290467/88610"/>
-    <hyperlink ref="C52" r:id="rId51" display="https://a2is.ru/catalog/messendzhery-dlya-komandnoy-raboty/skrini"/>
-    <hyperlink ref="C53" r:id="rId52" display="https://www.iphones.ru/iNotes/mts-web-services-otkryla-besplatnyy-dostup-k-servisu-dlya-obmena-asinhronnymi-video"/>
-    <hyperlink ref="C54" r:id="rId53" display="https://vc.ru/services/3041069-konstruktor-saytov-svadb-privlecheniy"/>
-    <hyperlink ref="C55" r:id="rId54" display="https://www.rustore.ru/catalog/app/ru.komod.app"/>
-    <hyperlink ref="C56" r:id="rId55" display="https://www.rustore.ru/catalog/app/click.opora.app"/>
-  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>